<commit_message>
progress: 22 village workbooks (sivaramans-llin 2026-10-09T10:10:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Old_Gummidipoondi_13.406625_80.12876.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Old_Gummidipoondi_13.406625_80.12876.xlsx
@@ -782,6 +782,11 @@
           <t>125</t>
         </is>
       </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C1, 2C2A, 2C2B, 2C2C, 2C2D, 2C2E, 2D</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -789,6 +794,11 @@
           <t>126</t>
         </is>
       </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -796,6 +806,11 @@
           <t>127</t>
         </is>
       </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -803,6 +818,11 @@
           <t>128</t>
         </is>
       </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -810,6 +830,11 @@
           <t>129</t>
         </is>
       </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1A1A1, 1A1B, 1A2A, 1A2B, 1A2C, 1A2D, 1A2E, 1A2F, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -817,6 +842,11 @@
           <t>13</t>
         </is>
       </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -824,6 +854,11 @@
           <t>130</t>
         </is>
       </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1B1, 1B2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -831,6 +866,11 @@
           <t>131</t>
         </is>
       </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -838,6 +878,11 @@
           <t>132</t>
         </is>
       </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1B1, 1B2, 1C, 1D, 2A1, 2A2A1, 2A2B, 2A2C, 2B1, 2B2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -845,6 +890,11 @@
           <t>133</t>
         </is>
       </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 3, 4A1, 4A2, 4B, 4C</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -852,6 +902,11 @@
           <t>134</t>
         </is>
       </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -859,6 +914,11 @@
           <t>135</t>
         </is>
       </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 3A, 3B1, 3B2, 3C1, 3C2, 4A, 4B, 5A, 5B, 5C, 5D, 5E</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -866,6 +926,11 @@
           <t>136</t>
         </is>
       </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 2E, 2F, 3A, 3B, 3C, 3D, 3E</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -873,6 +938,11 @@
           <t>137</t>
         </is>
       </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -880,6 +950,11 @@
           <t>138</t>
         </is>
       </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4A1, 4A2, 4A3, 4B1, 4B2, 4B3, 5, 6, 7, 8A, 8B1, 8B2</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -887,6 +962,11 @@
           <t>139</t>
         </is>
       </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -894,11 +974,21 @@
           <t>14</t>
         </is>
       </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A1C, 1A2, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
           <t>140</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2, 2B3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 23 village workbooks (randomwalk-TRX50-WS 2026-10-09T11:20:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Old_Gummidipoondi_13.406625_80.12876.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Old_Gummidipoondi_13.406625_80.12876.xlsx
@@ -4718,11 +4718,6 @@
           <t>41</t>
         </is>
       </c>
-      <c r="B359" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 3C, 4A, 4B, 4C, 5A, 5B, 5C</t>
-        </is>
-      </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -4730,11 +4725,6 @@
           <t>410</t>
         </is>
       </c>
-      <c r="B360" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -4742,11 +4732,6 @@
           <t>411</t>
         </is>
       </c>
-      <c r="B361" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2</t>
-        </is>
-      </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -4754,11 +4739,6 @@
           <t>412</t>
         </is>
       </c>
-      <c r="B362" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1B1A, 1B1B, 1B1C, 1B1D, 1B2, 2A1, 2A2, 2B, 3A1, 3A2, 3B, 4A, 4B, 4C1A1, 4C1A2, 4C1B1, 4C1B2, 4C2A, 4C2B1A1, 4C2B1A2, 4C2B1A3, 4C2B1A4, 4C2B1B, 4C2B2, 4C2B3A, 4C2B3B, 4C2B4A, 4C2B4B, 4C2B5A, 4C2B5B, 4C3A1, 4C3A2, 4C3B</t>
-        </is>
-      </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -4766,11 +4746,6 @@
           <t>413</t>
         </is>
       </c>
-      <c r="B363" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -4778,11 +4753,6 @@
           <t>414</t>
         </is>
       </c>
-      <c r="B364" t="inlineStr">
-        <is>
-          <t>10, 11A, 11B, 12, 13, 14, 15A, 15B1, 15B2, 15C, 16, 17A, 17B, 17C, 18, 19, 1A1, 1A2A, 1A2B1, 1B1A, 1B1B, 1B2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A1, 2A2, 2A3, 2A4, 2A5, 2A6A, 2A6B, 2A7, 2A8, 2B1, 2B2, 2B3, 2B4, 2B5, 2B6, 2B7, 2B8, 3A, 3B, 3C1A, 3C1B, 3C2, 4, 5A1A, 5A1B, 5A1C, 5A1D, 5A2, 5B, 6A1, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -4790,11 +4760,6 @@
           <t>415</t>
         </is>
       </c>
-      <c r="B365" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1B1A, 1B1B, 1B2, 1B3A, 1B3B, 1B3C, 1B4, 1B5, 1B6A1, 1B6A2A, 1B6A2B, 1B6B, 1B7A, 1B7B, 1C, 2A, 2B, 3A, 3B1, 3B2, 4A, 4B, 4C, 4D, 4E, 4F1, 4F2</t>
-        </is>
-      </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -4802,11 +4767,6 @@
           <t>416</t>
         </is>
       </c>
-      <c r="B366" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4A, 4B, 4C</t>
-        </is>
-      </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -4814,11 +4774,6 @@
           <t>417</t>
         </is>
       </c>
-      <c r="B367" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5A, 5B, 5C, 6</t>
-        </is>
-      </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -4826,11 +4781,6 @@
           <t>418</t>
         </is>
       </c>
-      <c r="B368" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1A3, 1B1A, 1B1B, 1B2A, 1B2B, 1B2C, 1B3, 1B4A, 1B4B, 1B4C, 1B5A, 1B5B, 2A, 2B, 2C, 2D1, 2D2, 2E1, 2E2, 2F, 2G1, 2G2, 2G3, 2H1, 2H2, 2I, 2J</t>
-        </is>
-      </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -4838,11 +4788,6 @@
           <t>419</t>
         </is>
       </c>
-      <c r="B369" t="inlineStr">
-        <is>
-          <t>1A, 1B10, 1B11A1, 1B11B, 1B11C, 1B11D, 1B1A, 1B1B, 1B1C, 1B2A, 1B2B, 1B3A1, 1B3A2, 1B3B, 1B3C, 1B4, 1B5, 1B6, 1B7A, 1B7B, 1B7C, 1B7D, 1B8A, 1B8B, 1B9, 1C, 2A1, 2A2, 2B, 2C, 3A1, 3A2, 3B, 4A1, 4A2, 4B1, 4B2, 4C, 4D</t>
-        </is>
-      </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
@@ -4850,11 +4795,6 @@
           <t>42</t>
         </is>
       </c>
-      <c r="B370" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 2C</t>
-        </is>
-      </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
@@ -4862,11 +4802,6 @@
           <t>420</t>
         </is>
       </c>
-      <c r="B371" t="inlineStr">
-        <is>
-          <t>1A, 1B1, 1B2, 1B3, 1C, 2</t>
-        </is>
-      </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
@@ -4874,11 +4809,6 @@
           <t>421</t>
         </is>
       </c>
-      <c r="B372" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 2C, 3A, 3B, 3C, 4, 5A, 5B</t>
-        </is>
-      </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
@@ -4886,11 +4816,6 @@
           <t>422</t>
         </is>
       </c>
-      <c r="B373" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 1D, 2A, 2B, 2C, 3A, 3B, 3C, 3D, 4A, 4B, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
@@ -4898,11 +4823,6 @@
           <t>423</t>
         </is>
       </c>
-      <c r="B374" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
@@ -4910,11 +4830,6 @@
           <t>424</t>
         </is>
       </c>
-      <c r="B375" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1A3, 1B1, 1B2, 2A, 2B1, 2B2</t>
-        </is>
-      </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
@@ -4922,11 +4837,6 @@
           <t>425</t>
         </is>
       </c>
-      <c r="B376" t="inlineStr">
-        <is>
-          <t>1, 2A1, 2A2, 2B</t>
-        </is>
-      </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
@@ -4934,11 +4844,6 @@
           <t>426</t>
         </is>
       </c>
-      <c r="B377" t="inlineStr">
-        <is>
-          <t>1A, 1B1, 1B2, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
@@ -4946,11 +4851,6 @@
           <t>427</t>
         </is>
       </c>
-      <c r="B378" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
@@ -4958,11 +4858,6 @@
           <t>428</t>
         </is>
       </c>
-      <c r="B379" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
@@ -4970,11 +4865,6 @@
           <t>429</t>
         </is>
       </c>
-      <c r="B380" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
@@ -4982,11 +4872,6 @@
           <t>43</t>
         </is>
       </c>
-      <c r="B381" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
@@ -4994,11 +4879,6 @@
           <t>430</t>
         </is>
       </c>
-      <c r="B382" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
@@ -5006,11 +4886,6 @@
           <t>431</t>
         </is>
       </c>
-      <c r="B383" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
@@ -5018,11 +4893,6 @@
           <t>432</t>
         </is>
       </c>
-      <c r="B384" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3A, 3B</t>
-        </is>
-      </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
@@ -5030,11 +4900,6 @@
           <t>433</t>
         </is>
       </c>
-      <c r="B385" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
@@ -5042,11 +4907,6 @@
           <t>434</t>
         </is>
       </c>
-      <c r="B386" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
@@ -5054,11 +4914,6 @@
           <t>435</t>
         </is>
       </c>
-      <c r="B387" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
@@ -5066,11 +4921,6 @@
           <t>436</t>
         </is>
       </c>
-      <c r="B388" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1A3, 1A4, 1B, 2</t>
-        </is>
-      </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
@@ -5078,11 +4928,6 @@
           <t>437</t>
         </is>
       </c>
-      <c r="B389" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
@@ -5090,11 +4935,6 @@
           <t>438</t>
         </is>
       </c>
-      <c r="B390" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
@@ -5102,11 +4942,6 @@
           <t>439</t>
         </is>
       </c>
-      <c r="B391" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
@@ -5114,11 +4949,6 @@
           <t>44</t>
         </is>
       </c>
-      <c r="B392" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
@@ -5126,11 +4956,6 @@
           <t>440</t>
         </is>
       </c>
-      <c r="B393" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
@@ -5138,11 +4963,6 @@
           <t>441</t>
         </is>
       </c>
-      <c r="B394" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 3C1A, 3C1B, 3C2, 3D, 3E1, 3E2</t>
-        </is>
-      </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
@@ -5150,11 +4970,6 @@
           <t>442</t>
         </is>
       </c>
-      <c r="B395" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
@@ -5162,11 +4977,6 @@
           <t>443</t>
         </is>
       </c>
-      <c r="B396" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
@@ -5174,11 +4984,6 @@
           <t>444</t>
         </is>
       </c>
-      <c r="B397" t="inlineStr">
-        <is>
-          <t>1A1, 1A2A, 1A2B, 1B, 2, 3, 4A, 4B, 4C, 5A1, 5A2, 5A3, 5B1, 5B2, 6A1A, 6A2, 6A3, 6A4, 6B, 7, 8A1, 8A2A1, 8A2A2, 8A2B, 8A2C, 8B1A, 8B1B, 8B2</t>
-        </is>
-      </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
@@ -5186,11 +4991,6 @@
           <t>445</t>
         </is>
       </c>
-      <c r="B398" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
@@ -5198,11 +4998,6 @@
           <t>446</t>
         </is>
       </c>
-      <c r="B399" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1B, 2A, 2B, 3A, 3B, 3C</t>
-        </is>
-      </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
@@ -5210,11 +5005,6 @@
           <t>447</t>
         </is>
       </c>
-      <c r="B400" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13, 14, 15, 16A, 16B, 17A, 17B, 18A, 18B, 19, 1A, 1B, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A, 2B, 3, 30, 31, 32, 33A, 33B, 34, 35A, 35B, 36, 37, 38, 39, 4, 40, 41, 42A, 42B, 5, 6, 7A, 7B, 8A, 8B, 8C, 9</t>
-        </is>
-      </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
@@ -5222,11 +5012,6 @@
           <t>448</t>
         </is>
       </c>
-      <c r="B401" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
@@ -5234,11 +5019,6 @@
           <t>449</t>
         </is>
       </c>
-      <c r="B402" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2</t>
-        </is>
-      </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
@@ -5246,11 +5026,6 @@
           <t>45</t>
         </is>
       </c>
-      <c r="B403" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
@@ -5258,11 +5033,6 @@
           <t>450</t>
         </is>
       </c>
-      <c r="B404" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
@@ -5270,11 +5040,6 @@
           <t>451</t>
         </is>
       </c>
-      <c r="B405" t="inlineStr">
-        <is>
-          <t>1A, 1B1, 1B2, 1C, 2A, 2B, 3</t>
-        </is>
-      </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
@@ -5282,11 +5047,6 @@
           <t>452</t>
         </is>
       </c>
-      <c r="B406" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
@@ -5294,11 +5054,6 @@
           <t>453</t>
         </is>
       </c>
-      <c r="B407" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 2C</t>
-        </is>
-      </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
@@ -5306,11 +5061,6 @@
           <t>454</t>
         </is>
       </c>
-      <c r="B408" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1A3, 1B, 1C, 1D, 2A, 2B, 2C</t>
-        </is>
-      </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
@@ -5318,11 +5068,6 @@
           <t>455</t>
         </is>
       </c>
-      <c r="B409" t="inlineStr">
-        <is>
-          <t>10, 1A1A1A1A, 1A1A2, 1A1A3, 1A1B, 1A2, 1A3, 1B, 2A, 2B, 2C, 3A1, 3A2A, 3A2B, 3B, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
@@ -5330,11 +5075,6 @@
           <t>456</t>
         </is>
       </c>
-      <c r="B410" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
@@ -5342,11 +5082,6 @@
           <t>457</t>
         </is>
       </c>
-      <c r="B411" t="inlineStr">
-        <is>
-          <t>10, 11, 1A1A, 1A2, 1A3, 1B, 2A, 2B, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
@@ -5354,11 +5089,6 @@
           <t>458</t>
         </is>
       </c>
-      <c r="B412" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
@@ -5366,11 +5096,6 @@
           <t>459</t>
         </is>
       </c>
-      <c r="B413" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
@@ -5378,11 +5103,6 @@
           <t>46</t>
         </is>
       </c>
-      <c r="B414" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
@@ -5390,11 +5110,6 @@
           <t>460</t>
         </is>
       </c>
-      <c r="B415" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1B, 1C, 2A1, 2A2, 2B, 3A1, 3B, 3C, 4A, 4B, 5, 6, 7A, 7B</t>
-        </is>
-      </c>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
@@ -5402,11 +5117,6 @@
           <t>461</t>
         </is>
       </c>
-      <c r="B416" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
@@ -5414,11 +5124,6 @@
           <t>462</t>
         </is>
       </c>
-      <c r="B417" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A1, 2A2, 2B1, 2B2, 2C, 2D, 3A, 3B</t>
-        </is>
-      </c>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
@@ -5426,11 +5131,6 @@
           <t>463</t>
         </is>
       </c>
-      <c r="B418" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 2</t>
-        </is>
-      </c>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
@@ -5438,11 +5138,6 @@
           <t>464</t>
         </is>
       </c>
-      <c r="B419" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A1A1, 2A1A2, 2A1A3, 2A1A4, 2A1B, 2A1C, 2A2A, 2A2B, 2A2C, 2B1, 2B2</t>
-        </is>
-      </c>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
@@ -5450,11 +5145,6 @@
           <t>465</t>
         </is>
       </c>
-      <c r="B420" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A, 2B, 2C1, 2C2A, 2C2B</t>
-        </is>
-      </c>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
@@ -5462,11 +5152,6 @@
           <t>466</t>
         </is>
       </c>
-      <c r="B421" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
@@ -5474,11 +5159,6 @@
           <t>467</t>
         </is>
       </c>
-      <c r="B422" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
@@ -5486,11 +5166,6 @@
           <t>468</t>
         </is>
       </c>
-      <c r="B423" t="inlineStr">
-        <is>
-          <t>1A, 1B1A, 1B1B, 1B2, 2</t>
-        </is>
-      </c>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
@@ -5498,11 +5173,6 @@
           <t>469</t>
         </is>
       </c>
-      <c r="B424" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1A3, 1A4, 1A5, 1A6, 1A7, 1A8, 1B, 2A1, 2A2, 2A3, 2A4, 2B1, 2B2, 2B3, 2B4A, 2B4B, 2C, 2D1, 2D2, 2D3, 3A, 3B, 4A, 4B1, 4B2A1A, 4B2A2, 4B2B, 4B3, 5A1A1, 5A2, 5A3, 5B, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
@@ -5510,11 +5180,6 @@
           <t>47</t>
         </is>
       </c>
-      <c r="B425" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="426">
       <c r="A426" t="inlineStr">
@@ -5522,11 +5187,6 @@
           <t>470</t>
         </is>
       </c>
-      <c r="B426" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
@@ -5534,11 +5194,6 @@
           <t>471</t>
         </is>
       </c>
-      <c r="B427" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A, 2B, 3A, 3B</t>
-        </is>
-      </c>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
@@ -5546,11 +5201,6 @@
           <t>472</t>
         </is>
       </c>
-      <c r="B428" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
@@ -5558,11 +5208,6 @@
           <t>473</t>
         </is>
       </c>
-      <c r="B429" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
@@ -5570,11 +5215,6 @@
           <t>474</t>
         </is>
       </c>
-      <c r="B430" t="inlineStr">
-        <is>
-          <t>1, 10, 100, 101, 102, 103, 104, 105, 106, 107, 108, 109, 11, 110, 111, 112, 113, 114, 115, 116, 117, 118, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 3, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 4, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 5, 50, 51, 52, 53, 54, 55, 56, 57, 58, 59, 6, 60, 61, 62, 63, 64, 65, 66, 67, 68, 69, 70, 71, 72, 73, 74, 75, 76, 77, 78, 79, 7A, 7B, 8, 80, 81, 82, 83, 84, 85, 86, 87, 88, 89, 9, 90, 91, 92, 93, 94, 95, 96, 97, 98, 99</t>
-        </is>
-      </c>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
@@ -5582,11 +5222,6 @@
           <t>475</t>
         </is>
       </c>
-      <c r="B431" t="inlineStr">
-        <is>
-          <t>1, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A1, 2A2, 2A3, 2B1, 2B10, 2B11, 2B12, 2B13, 2B14, 2B15, 2B16, 2B17A, 2B17B, 2B18A, 2B18B, 2B18C, 2B19, 2B2, 2B3, 2B4, 2B5, 2B6, 2B7, 2B8, 2B9, 2C1A1, 2C1B, 2C2A1, 2C2A2, 2C2B, 2C3, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 50, 51, 52, 53, 54, 55, 56, 57, 58, 59, 60, 61, 62, 63, 64, 65, 66, 67, 68, 69, 70, 71, 72, 73, 74, 75, 76, 77, 78, 79, 80, 81, 82, 83, 84, 85, 86</t>
-        </is>
-      </c>
     </row>
     <row r="432">
       <c r="A432" t="inlineStr">
@@ -5594,11 +5229,6 @@
           <t>476</t>
         </is>
       </c>
-      <c r="B432" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="433">
       <c r="A433" t="inlineStr">
@@ -5606,11 +5236,6 @@
           <t>477</t>
         </is>
       </c>
-      <c r="B433" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1B, 2A, 2B</t>
-        </is>
-      </c>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
@@ -5618,11 +5243,6 @@
           <t>478</t>
         </is>
       </c>
-      <c r="B434" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
@@ -5630,11 +5250,6 @@
           <t>479</t>
         </is>
       </c>
-      <c r="B435" t="inlineStr">
-        <is>
-          <t>1, 21, 2A1, 2A2, 2B1A1A, 2B1A1B, 2B1A2A, 2B1A2B, 2B1A2C, 2B1A2D, 2B1A2E, 2B1B, 2B2, 4A, 4B, 4C, 4D, 5B1, 5B2, 5B3, 5B4, 6, 7A1A1, 7A1A2A, 7A1A2B, 7A1B, 7A2, 7A2A1, 7A2A2, 7A2A3, 7A2A4, 7A2B1, 7A2B10, 7A2B12, 7A2B13, 7A2B14, 7A2B15A1, 7A2B2A, 7A2B2B, 7A2B3, 7A2B4, 7A2B5, 7A2B6, 7A2B7A, 7A2B7B, 7A2B8A, 7A2B8B, 7A2B9, 7B1A, 7B1B, 7B2A, 7B2B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="436">
       <c r="A436" t="inlineStr">
@@ -5642,11 +5257,6 @@
           <t>48</t>
         </is>
       </c>
-      <c r="B436" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A, 2B, 3, 4A, 4B, 5</t>
-        </is>
-      </c>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
@@ -5654,11 +5264,6 @@
           <t>480</t>
         </is>
       </c>
-      <c r="B437" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3A, 3B</t>
-        </is>
-      </c>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
@@ -5666,11 +5271,6 @@
           <t>481</t>
         </is>
       </c>
-      <c r="B438" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B1, 2B2</t>
-        </is>
-      </c>
     </row>
     <row r="439">
       <c r="A439" t="inlineStr">
@@ -5678,11 +5278,6 @@
           <t>482</t>
         </is>
       </c>
-      <c r="B439" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
@@ -5690,11 +5285,6 @@
           <t>483</t>
         </is>
       </c>
-      <c r="B440" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 19, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A, 2B, 2C, 30, 31, 3A1A1, 3A1B, 3A2, 3B, 4A, 4B1, 4B2A1A, 5A1, 5A1B, 5A1C1A, 5A1C2, 5A2, 5B1A, 5B1B, 5B1C, 5B2, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="441">
       <c r="A441" t="inlineStr">
@@ -5702,11 +5292,6 @@
           <t>484</t>
         </is>
       </c>
-      <c r="B441" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
@@ -5714,11 +5299,6 @@
           <t>485</t>
         </is>
       </c>
-      <c r="B442" t="inlineStr">
-        <is>
-          <t>1, 1A1, 1A2A, 1A2B, 1A2C, 1A3, 1B1, 1B2, 1B3, 1C1, 1C2A, 1C2B, 1C2C, 1D1, 1D2A1, 1D2A2, 1D2B, 1D2C, 1D2D, 1D2E, 1E1, 1E2A, 1E2B, 1E2C, 1E3, 1F, 2</t>
-        </is>
-      </c>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
@@ -5726,11 +5306,6 @@
           <t>486</t>
         </is>
       </c>
-      <c r="B443" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
@@ -5738,11 +5313,6 @@
           <t>487</t>
         </is>
       </c>
-      <c r="B444" t="inlineStr">
-        <is>
-          <t>10, 11, 12A, 12B, 1A1A1, 1B, 1C, 1D, 1E, 1F, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
@@ -5750,11 +5320,6 @@
           <t>488</t>
         </is>
       </c>
-      <c r="B445" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
@@ -5762,11 +5327,6 @@
           <t>489</t>
         </is>
       </c>
-      <c r="B446" t="inlineStr">
-        <is>
-          <t>1A1, 1A2A, 1A2B1, 1A2B2, 1B, 1C1, 1C2, 2A, 2B</t>
-        </is>
-      </c>
     </row>
     <row r="447">
       <c r="A447" t="inlineStr">
@@ -5774,11 +5334,6 @@
           <t>49</t>
         </is>
       </c>
-      <c r="B447" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1B, 1C, 1D, 2</t>
-        </is>
-      </c>
     </row>
     <row r="448">
       <c r="A448" t="inlineStr">
@@ -5786,11 +5341,6 @@
           <t>490</t>
         </is>
       </c>
-      <c r="B448" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="449">
       <c r="A449" t="inlineStr">
@@ -5798,11 +5348,6 @@
           <t>491</t>
         </is>
       </c>
-      <c r="B449" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="450">
       <c r="A450" t="inlineStr">
@@ -5810,11 +5355,6 @@
           <t>492</t>
         </is>
       </c>
-      <c r="B450" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="451">
       <c r="A451" t="inlineStr">
@@ -5822,11 +5362,6 @@
           <t>493</t>
         </is>
       </c>
-      <c r="B451" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
@@ -5834,11 +5369,6 @@
           <t>494</t>
         </is>
       </c>
-      <c r="B452" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
@@ -5846,11 +5376,6 @@
           <t>495</t>
         </is>
       </c>
-      <c r="B453" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
@@ -5858,11 +5383,6 @@
           <t>496</t>
         </is>
       </c>
-      <c r="B454" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 2C, 3A, 3B, 4, 5, 6A, 6B, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
@@ -5870,11 +5390,6 @@
           <t>497</t>
         </is>
       </c>
-      <c r="B455" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7, 8A, 8B</t>
-        </is>
-      </c>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
@@ -5882,11 +5397,6 @@
           <t>498A</t>
         </is>
       </c>
-      <c r="B456" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="457">
       <c r="A457" t="inlineStr">
@@ -5894,11 +5404,6 @@
           <t>498B</t>
         </is>
       </c>
-      <c r="B457" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="458">
       <c r="A458" t="inlineStr">
@@ -5906,11 +5411,6 @@
           <t>499</t>
         </is>
       </c>
-      <c r="B458" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="459">
       <c r="A459" t="inlineStr">
@@ -5918,11 +5418,6 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B459" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
@@ -5930,11 +5425,6 @@
           <t>50</t>
         </is>
       </c>
-      <c r="B460" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
@@ -5942,11 +5432,6 @@
           <t>500A</t>
         </is>
       </c>
-      <c r="B461" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="462">
       <c r="A462" t="inlineStr">
@@ -5954,11 +5439,6 @@
           <t>500B</t>
         </is>
       </c>
-      <c r="B462" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="463">
       <c r="A463" t="inlineStr">
@@ -5966,11 +5446,6 @@
           <t>501</t>
         </is>
       </c>
-      <c r="B463" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="464">
       <c r="A464" t="inlineStr">
@@ -5978,11 +5453,6 @@
           <t>502</t>
         </is>
       </c>
-      <c r="B464" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1B, 2</t>
-        </is>
-      </c>
     </row>
     <row r="465">
       <c r="A465" t="inlineStr">
@@ -5990,11 +5460,6 @@
           <t>503A</t>
         </is>
       </c>
-      <c r="B465" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="466">
       <c r="A466" t="inlineStr">
@@ -6002,11 +5467,6 @@
           <t>503B</t>
         </is>
       </c>
-      <c r="B466" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="467">
       <c r="A467" t="inlineStr">
@@ -6014,11 +5474,6 @@
           <t>504A</t>
         </is>
       </c>
-      <c r="B467" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="468">
       <c r="A468" t="inlineStr">
@@ -6026,11 +5481,6 @@
           <t>504B</t>
         </is>
       </c>
-      <c r="B468" t="inlineStr">
-        <is>
-          <t>1, 2A1A, 2A1B, 2A1C, 2A2, 2B1, 2B2, 3A1, 3A2, 3A3, 3A4, 3A5, 3B</t>
-        </is>
-      </c>
     </row>
     <row r="469">
       <c r="A469" t="inlineStr">
@@ -6038,11 +5488,6 @@
           <t>505</t>
         </is>
       </c>
-      <c r="B469" t="inlineStr">
-        <is>
-          <t>1, 2A1, 2A2, 2B1, 2B2, 2C1, 2C2</t>
-        </is>
-      </c>
     </row>
     <row r="470">
       <c r="A470" t="inlineStr">
@@ -6050,11 +5495,6 @@
           <t>506A</t>
         </is>
       </c>
-      <c r="B470" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="471">
       <c r="A471" t="inlineStr">
@@ -6062,11 +5502,6 @@
           <t>506B</t>
         </is>
       </c>
-      <c r="B471" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="472">
       <c r="A472" t="inlineStr">
@@ -6074,11 +5509,6 @@
           <t>507</t>
         </is>
       </c>
-      <c r="B472" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="473">
       <c r="A473" t="inlineStr">
@@ -6086,11 +5516,6 @@
           <t>508</t>
         </is>
       </c>
-      <c r="B473" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="474">
       <c r="A474" t="inlineStr">
@@ -6098,11 +5523,6 @@
           <t>509</t>
         </is>
       </c>
-      <c r="B474" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 2A1A1A1, 2A1B, 2A2, 2A4, 2B, 2C, 3A15A1, 3A1A1, 3A1A2, 3A1B, 3A1C, 3A2, 3A3, 3A4A, 3A4B, 3A4C, 3A5A1B, 3A5A2, 3A5B, 3B, 4, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="475">
       <c r="A475" t="inlineStr">
@@ -6110,11 +5530,6 @@
           <t>51</t>
         </is>
       </c>
-      <c r="B475" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="476">
       <c r="A476" t="inlineStr">
@@ -6122,11 +5537,6 @@
           <t>510</t>
         </is>
       </c>
-      <c r="B476" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="477">
       <c r="A477" t="inlineStr">
@@ -6134,11 +5544,6 @@
           <t>511</t>
         </is>
       </c>
-      <c r="B477" t="inlineStr">
-        <is>
-          <t>1A1A, 1A1B, 1A2A, 1A2B, 1B1A1, 1B1A2, 1B1A3, 1B1B, 1B2, 1B3, 2A, 2B1, 2B2, 3A, 3B1A1, 3B1A2A1, 3B1A2A2, 3B1B, 3B2A, 3B2B, 4A, 4B, 5, 6, 7, 8A, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="478">
       <c r="A478" t="inlineStr">
@@ -6146,11 +5551,6 @@
           <t>512</t>
         </is>
       </c>
-      <c r="B478" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1B1, 1B2, 2</t>
-        </is>
-      </c>
     </row>
     <row r="479">
       <c r="A479" t="inlineStr">
@@ -6158,11 +5558,6 @@
           <t>514</t>
         </is>
       </c>
-      <c r="B479" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="480">
       <c r="A480" t="inlineStr">
@@ -6170,11 +5565,6 @@
           <t>516</t>
         </is>
       </c>
-      <c r="B480" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="481">
       <c r="A481" t="inlineStr">
@@ -6182,11 +5572,6 @@
           <t>517</t>
         </is>
       </c>
-      <c r="B481" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="482">
       <c r="A482" t="inlineStr">
@@ -6194,11 +5579,6 @@
           <t>52</t>
         </is>
       </c>
-      <c r="B482" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="483">
       <c r="A483" t="inlineStr">
@@ -6206,11 +5586,6 @@
           <t>522</t>
         </is>
       </c>
-      <c r="B483" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="484">
       <c r="A484" t="inlineStr">
@@ -6218,11 +5593,6 @@
           <t>523</t>
         </is>
       </c>
-      <c r="B484" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="485">
       <c r="A485" t="inlineStr">
@@ -6230,11 +5600,6 @@
           <t>524</t>
         </is>
       </c>
-      <c r="B485" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="486">
       <c r="A486" t="inlineStr">
@@ -6242,11 +5607,6 @@
           <t>525</t>
         </is>
       </c>
-      <c r="B486" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="487">
       <c r="A487" t="inlineStr">
@@ -6254,11 +5614,6 @@
           <t>526</t>
         </is>
       </c>
-      <c r="B487" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="488">
       <c r="A488" t="inlineStr">
@@ -6266,11 +5621,6 @@
           <t>527</t>
         </is>
       </c>
-      <c r="B488" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="489">
       <c r="A489" t="inlineStr">
@@ -6278,11 +5628,6 @@
           <t>528A</t>
         </is>
       </c>
-      <c r="B489" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2</t>
-        </is>
-      </c>
     </row>
     <row r="490">
       <c r="A490" t="inlineStr">
@@ -6290,11 +5635,6 @@
           <t>528B</t>
         </is>
       </c>
-      <c r="B490" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="491">
       <c r="A491" t="inlineStr">
@@ -6302,11 +5642,6 @@
           <t>529A</t>
         </is>
       </c>
-      <c r="B491" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="492">
       <c r="A492" t="inlineStr">
@@ -6314,11 +5649,6 @@
           <t>529B</t>
         </is>
       </c>
-      <c r="B492" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="493">
       <c r="A493" t="inlineStr">
@@ -6326,11 +5656,6 @@
           <t>53</t>
         </is>
       </c>
-      <c r="B493" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2</t>
-        </is>
-      </c>
     </row>
     <row r="494">
       <c r="A494" t="inlineStr">
@@ -6338,11 +5663,6 @@
           <t>530A</t>
         </is>
       </c>
-      <c r="B494" t="inlineStr">
-        <is>
-          <t>1A1A, 1A1B, 1A2, 1A3A, 1A3B, 1B, 2</t>
-        </is>
-      </c>
     </row>
     <row r="495">
       <c r="A495" t="inlineStr">
@@ -6350,11 +5670,6 @@
           <t>530B</t>
         </is>
       </c>
-      <c r="B495" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 2C</t>
-        </is>
-      </c>
     </row>
     <row r="496">
       <c r="A496" t="inlineStr">
@@ -6362,11 +5677,6 @@
           <t>531</t>
         </is>
       </c>
-      <c r="B496" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B1, 2B2A, 2B2B, 2B2C</t>
-        </is>
-      </c>
     </row>
     <row r="497">
       <c r="A497" t="inlineStr">
@@ -6374,11 +5684,6 @@
           <t>532A</t>
         </is>
       </c>
-      <c r="B497" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B1A, 3B1B, 3B2A, 3B2B, 4, 5A, 5B</t>
-        </is>
-      </c>
     </row>
     <row r="498">
       <c r="A498" t="inlineStr">
@@ -6386,11 +5691,6 @@
           <t>532B</t>
         </is>
       </c>
-      <c r="B498" t="inlineStr">
-        <is>
-          <t>1, 2A1, 2A2A, 2A2B, 2A2C, 2A3, 2A4A, 2A4B, 2A4C, 2A4D, 2B1A, 2B1B, 2B1C, 2B2A, 2B2B, 2C1, 2C2</t>
-        </is>
-      </c>
     </row>
     <row r="499">
       <c r="A499" t="inlineStr">
@@ -6398,11 +5698,6 @@
           <t>533</t>
         </is>
       </c>
-      <c r="B499" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="500">
       <c r="A500" t="inlineStr">
@@ -6410,11 +5705,6 @@
           <t>534</t>
         </is>
       </c>
-      <c r="B500" t="inlineStr">
-        <is>
-          <t>1A, 1B1, 1B2, 1B3, 2A, 2B1, 2B2, 3A, 3B1A1, 3B1A2, 3B1B, 3B2, 4</t>
-        </is>
-      </c>
     </row>
     <row r="501">
       <c r="A501" t="inlineStr">
@@ -6422,11 +5712,6 @@
           <t>535</t>
         </is>
       </c>
-      <c r="B501" t="inlineStr">
-        <is>
-          <t>1A, 1B1, 1B2, 2A, 2B, 3A1, 3A2, 3B, 4, 5, 6A, 6B, 6C, 6D, 6E, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="502">
       <c r="A502" t="inlineStr">
@@ -6434,11 +5719,6 @@
           <t>536</t>
         </is>
       </c>
-      <c r="B502" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 1D, 1E, 1F, 2</t>
-        </is>
-      </c>
     </row>
     <row r="503">
       <c r="A503" t="inlineStr">
@@ -6446,11 +5726,6 @@
           <t>537</t>
         </is>
       </c>
-      <c r="B503" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2</t>
-        </is>
-      </c>
     </row>
     <row r="504">
       <c r="A504" t="inlineStr">
@@ -6458,11 +5733,6 @@
           <t>538</t>
         </is>
       </c>
-      <c r="B504" t="inlineStr">
-        <is>
-          <t>10, 1A1, 1A2, 1A3, 1A4, 1A5, 1A6, 1B, 1C, 1D, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="505">
       <c r="A505" t="inlineStr">
@@ -6470,11 +5740,6 @@
           <t>539</t>
         </is>
       </c>
-      <c r="B505" t="inlineStr">
-        <is>
-          <t>1TO5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="506">
       <c r="A506" t="inlineStr">
@@ -6482,11 +5747,6 @@
           <t>54</t>
         </is>
       </c>
-      <c r="B506" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G1, 1G2, 2</t>
-        </is>
-      </c>
     </row>
     <row r="507">
       <c r="A507" t="inlineStr">
@@ -6494,11 +5754,6 @@
           <t>540</t>
         </is>
       </c>
-      <c r="B507" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="508">
       <c r="A508" t="inlineStr">
@@ -6506,11 +5761,6 @@
           <t>541A</t>
         </is>
       </c>
-      <c r="B508" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3, 4, 5, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="509">
       <c r="A509" t="inlineStr">
@@ -6518,11 +5768,6 @@
           <t>541B</t>
         </is>
       </c>
-      <c r="B509" t="inlineStr">
-        <is>
-          <t>1, 2A1, 2A2, 2A3, 2A4, 2A5, 2B, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="510">
       <c r="A510" t="inlineStr">
@@ -6530,11 +5775,6 @@
           <t>542A</t>
         </is>
       </c>
-      <c r="B510" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A1, 1A2, 1D, 2, 20, 21, 22, 23, 24, 25, 26, 3A1, 3A2A1, 3A2B1, 3B1A, 3B1A1, 3B1B1A2, 3B1B1B, 3B1B2, 3B2A1A, 3B2A1B, 3B2A2A, 3B2A3A1, 3B2A3B, 3B2B, 3B2C1A, 3B2C1B, 3B2C2A, 3B2C2B, 4, 5, 6A1, 6A2, 6B, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="511">
       <c r="A511" t="inlineStr">
@@ -6542,11 +5782,6 @@
           <t>542B</t>
         </is>
       </c>
-      <c r="B511" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="512">
       <c r="A512" t="inlineStr">
@@ -6554,11 +5789,6 @@
           <t>543</t>
         </is>
       </c>
-      <c r="B512" t="inlineStr">
-        <is>
-          <t>1, 2, 3A1A, 3A1B, 3A2, 3B</t>
-        </is>
-      </c>
     </row>
     <row r="513">
       <c r="A513" t="inlineStr">
@@ -6566,11 +5796,6 @@
           <t>544</t>
         </is>
       </c>
-      <c r="B513" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13, 14, 15A1, 15A2, 15B, 16, 17, 18, 1A1, 1A2, 1B, 2A, 2B1, 2B2, 2B3, 3, 4A1A, 4A1B, 4A1C, 4A1D1, 4A1D2, 4A2, 4A3, 4B1A1A, 4B1A2, 4B1B, 4B2, 5A1A1, 5A1A1A1A1, 5A1A1A1B, 5A1A1B2, 5A1A2A, 5A1A2B, 5A1A3, 5A1B, 5A2A1, 5A2B, 5B1, 5B2, 6, 7A, 7B, 7C1, 7C2, 8A, 8B, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="514">
       <c r="A514" t="inlineStr">
@@ -6578,11 +5803,6 @@
           <t>545</t>
         </is>
       </c>
-      <c r="B514" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B1A1, 2B1A2, 2B1A3, 2B1B, 2B2, 3A1A, 3A1B, 3A1C, 3A1D, 3A2, 3A3, 3A4, 3A5, 3A6, 3B</t>
-        </is>
-      </c>
     </row>
     <row r="515">
       <c r="A515" t="inlineStr">
@@ -6590,11 +5810,6 @@
           <t>546</t>
         </is>
       </c>
-      <c r="B515" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="516">
       <c r="A516" t="inlineStr">
@@ -6602,11 +5817,6 @@
           <t>547A</t>
         </is>
       </c>
-      <c r="B516" t="inlineStr">
-        <is>
-          <t>1, 10, 2A, 2B, 3A, 3B, 4, 5A, 5B, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="517">
       <c r="A517" t="inlineStr">
@@ -6614,11 +5824,6 @@
           <t>547B</t>
         </is>
       </c>
-      <c r="B517" t="inlineStr">
-        <is>
-          <t>1, 2A1, 2A2, 2B, 3</t>
-        </is>
-      </c>
     </row>
     <row r="518">
       <c r="A518" t="inlineStr">
@@ -6626,11 +5831,6 @@
           <t>548</t>
         </is>
       </c>
-      <c r="B518" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3A1, 3A2, 3B, 3C, 4, 5A1, 5A2, 5B</t>
-        </is>
-      </c>
     </row>
     <row r="519">
       <c r="A519" t="inlineStr">
@@ -6638,11 +5838,6 @@
           <t>549</t>
         </is>
       </c>
-      <c r="B519" t="inlineStr">
-        <is>
-          <t>1, 2A1A1, 2A1A2, 2A1B, 2A2, 2A3, 2B</t>
-        </is>
-      </c>
     </row>
     <row r="520">
       <c r="A520" t="inlineStr">
@@ -6650,11 +5845,6 @@
           <t>55</t>
         </is>
       </c>
-      <c r="B520" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="521">
       <c r="A521" t="inlineStr">
@@ -6662,11 +5852,6 @@
           <t>550</t>
         </is>
       </c>
-      <c r="B521" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="522">
       <c r="A522" t="inlineStr">
@@ -6674,11 +5859,6 @@
           <t>551</t>
         </is>
       </c>
-      <c r="B522" t="inlineStr">
-        <is>
-          <t>1, 2, 3A1A, 3A1B1, 3A1B2, 3A2A, 3A2B, 3B, 4</t>
-        </is>
-      </c>
     </row>
     <row r="523">
       <c r="A523" t="inlineStr">
@@ -6686,11 +5866,6 @@
           <t>552A</t>
         </is>
       </c>
-      <c r="B523" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="524">
       <c r="A524" t="inlineStr">
@@ -6698,11 +5873,6 @@
           <t>552B</t>
         </is>
       </c>
-      <c r="B524" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="525">
       <c r="A525" t="inlineStr">
@@ -6710,11 +5880,6 @@
           <t>553A</t>
         </is>
       </c>
-      <c r="B525" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="526">
       <c r="A526" t="inlineStr">
@@ -6722,11 +5887,6 @@
           <t>553B</t>
         </is>
       </c>
-      <c r="B526" t="inlineStr">
-        <is>
-          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="527">
       <c r="A527" t="inlineStr">
@@ -6734,11 +5894,6 @@
           <t>554</t>
         </is>
       </c>
-      <c r="B527" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="528">
       <c r="A528" t="inlineStr">
@@ -6746,11 +5901,6 @@
           <t>555</t>
         </is>
       </c>
-      <c r="B528" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="529">
       <c r="A529" t="inlineStr">
@@ -6758,11 +5908,6 @@
           <t>556</t>
         </is>
       </c>
-      <c r="B529" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="530">
       <c r="A530" t="inlineStr">
@@ -6770,11 +5915,6 @@
           <t>557</t>
         </is>
       </c>
-      <c r="B530" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="531">
       <c r="A531" t="inlineStr">
@@ -6782,11 +5922,6 @@
           <t>558</t>
         </is>
       </c>
-      <c r="B531" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="532">
       <c r="A532" t="inlineStr">
@@ -6794,11 +5929,6 @@
           <t>559A</t>
         </is>
       </c>
-      <c r="B532" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="533">
       <c r="A533" t="inlineStr">
@@ -6806,11 +5936,6 @@
           <t>559B</t>
         </is>
       </c>
-      <c r="B533" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="534">
       <c r="A534" t="inlineStr">
@@ -6818,11 +5943,6 @@
           <t>56</t>
         </is>
       </c>
-      <c r="B534" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="535">
       <c r="A535" t="inlineStr">
@@ -6830,11 +5950,6 @@
           <t>560A</t>
         </is>
       </c>
-      <c r="B535" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="536">
       <c r="A536" t="inlineStr">
@@ -6842,11 +5957,6 @@
           <t>560B</t>
         </is>
       </c>
-      <c r="B536" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="537">
       <c r="A537" t="inlineStr">
@@ -6854,11 +5964,6 @@
           <t>561</t>
         </is>
       </c>
-      <c r="B537" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="538">
       <c r="A538" t="inlineStr">
@@ -6866,11 +5971,6 @@
           <t>562</t>
         </is>
       </c>
-      <c r="B538" t="inlineStr">
-        <is>
-          <t>1, 10, 11A, 11B, 12A1A, 12A1B, 12A2, 12B, 13, 14, 15A, 15B, 15C, 15D, 16, 17A, 17B, 18, 19, 2, 20, 21A, 21B, 21C, 21D, 21E, 21F, 21G, 22, 23, 24A, 24B, 25A, 25B, 26A1, 26A2, 26B1, 26B2, 27A1A1, 27A1A2, 27A2, 27B1A, 27B1A2, 27B1A3, 27B1B, 27B1C, 27B2, 28, 29, 3, 30A1, 30A2, 30A3, 30A4, 30A5, 31, 32, 33, 34A1, 34A2, 34B, 34C, 35A, 35B, 36, 37, 38, 39, 42A, 42B, 43A, 43B1, 43B2, 44, 45, 46, 47, 48, 49, 4A, 4B, 4C, 4D, 4E, 4F, 4G, 5A, 5B, 5C, 5D, 5E, 6, 7, 8A, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="539">
       <c r="A539" t="inlineStr">
@@ -6878,11 +5978,6 @@
           <t>563</t>
         </is>
       </c>
-      <c r="B539" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 2A1A1, 2A1A2, 2A1B, 2A1C1A1, 2A1C2, 2A1C3A, 2A1C3B, 2A1C3C, 2A1C3D, 2A2A, 2A2B, 2B, 2C1, 2C2, 2C3, 2D1A1, 2D1A2, 2D1B1A, 2D1B1B, 2D1B2A, 2D2, 2E1, 2E2A1, 2E2A2, 2E2B, 3A1A1A, 3A1B, 3A1C, 3A1D, 3A1E, 3A1F, 3A2, 3A3A1, 3A3A2, 3A3A3, 3A3A4, 3A3B, 3A3C, 3B, 3C1A, 3C1A2, 3C1B, 3C1C, 3C1D, 3C2, 4, 40, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="540">
       <c r="A540" t="inlineStr">
@@ -6890,11 +5985,6 @@
           <t>564</t>
         </is>
       </c>
-      <c r="B540" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="541">
       <c r="A541" t="inlineStr">
@@ -6902,11 +5992,6 @@
           <t>565</t>
         </is>
       </c>
-      <c r="B541" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A1A, 2A1B, 2A1C, 2A2, 2B1A1A1, 2B1A1B, 2B1A2, 2B1A3, 2B1B, 2B2, 2B3A1, 2B3A2, 3, 4, 5, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="542">
       <c r="A542" t="inlineStr">
@@ -6914,11 +5999,6 @@
           <t>566</t>
         </is>
       </c>
-      <c r="B542" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="543">
       <c r="A543" t="inlineStr">
@@ -6926,11 +6006,6 @@
           <t>567</t>
         </is>
       </c>
-      <c r="B543" t="inlineStr">
-        <is>
-          <t>1, 2A1A, 2A1B, 2A2, 2A3, 2B1A, 2B1B, 2B2, 2C1, 2C2, 2C3</t>
-        </is>
-      </c>
     </row>
     <row r="544">
       <c r="A544" t="inlineStr">
@@ -6938,11 +6013,6 @@
           <t>568</t>
         </is>
       </c>
-      <c r="B544" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A, 2B</t>
-        </is>
-      </c>
     </row>
     <row r="545">
       <c r="A545" t="inlineStr">
@@ -6950,11 +6020,6 @@
           <t>569</t>
         </is>
       </c>
-      <c r="B545" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="546">
       <c r="A546" t="inlineStr">
@@ -6962,11 +6027,6 @@
           <t>57</t>
         </is>
       </c>
-      <c r="B546" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1A3, 1B, 1C, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="547">
       <c r="A547" t="inlineStr">
@@ -6974,11 +6034,6 @@
           <t>570</t>
         </is>
       </c>
-      <c r="B547" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="548">
       <c r="A548" t="inlineStr">
@@ -6986,11 +6041,6 @@
           <t>571</t>
         </is>
       </c>
-      <c r="B548" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="549">
       <c r="A549" t="inlineStr">
@@ -6998,11 +6048,6 @@
           <t>572</t>
         </is>
       </c>
-      <c r="B549" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A, 2B, 2C, 2D</t>
-        </is>
-      </c>
     </row>
     <row r="550">
       <c r="A550" t="inlineStr">
@@ -7010,11 +6055,6 @@
           <t>573</t>
         </is>
       </c>
-      <c r="B550" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A1A1A, 2A1A2, 2A1B, 2A2, 2B1, 2B2, 2C, 3A, 3B1, 3B2, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="551">
       <c r="A551" t="inlineStr">
@@ -7022,11 +6062,6 @@
           <t>574</t>
         </is>
       </c>
-      <c r="B551" t="inlineStr">
-        <is>
-          <t>1A1A, 1A1B, 1A2, 1B, 2A, 2B, 3A1A1, 3A1A2A, 3A1A2B, 3A1A3A, 3A1A3B, 3A1B, 3A2, 3B, 4A1A1, 4A1A2, 4A1B1A, 4A1B1B, 4A1B2, 4A2, 4B1A1, 4B1A2, 4B1B, 4B1C, 4B2A1, 4B2A2, 4B2B, 4C1, 4C2A, 4C2B, 4C3</t>
-        </is>
-      </c>
     </row>
     <row r="552">
       <c r="A552" t="inlineStr">
@@ -7034,11 +6069,6 @@
           <t>575</t>
         </is>
       </c>
-      <c r="B552" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="553">
       <c r="A553" t="inlineStr">
@@ -7046,11 +6076,6 @@
           <t>576</t>
         </is>
       </c>
-      <c r="B553" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="554">
       <c r="A554" t="inlineStr">
@@ -7058,11 +6083,6 @@
           <t>577</t>
         </is>
       </c>
-      <c r="B554" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13, 14, 15, 1A1A, 1A2A, 1A2B, 1B, 2A, 2B1A, 2B1A2, 2B1B, 2B2A, 2B2B, 2B2C, 2B2D1, 2B2D2, 2B2D3, 2B2D4, 3, 4A, 4B1, 4B2, 5A1, 5A2, 5B1A, 5B1B, 5B1C, 5B2A, 5B2B, 5B3A1, 5B3A2, 5B3B1, 5B3B2, 6A1A, 6A1B1, 6A1B2, 6A1B3, 6A2A, 6A2B, 6A2C1, 6A2C2, 6A2C3, 6A2D, 6A2E1, 6A2E2, 6A2E3, 6A2E4, 6A2E5, 6A2E6, 6A2E7, 6B, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="555">
       <c r="A555" t="inlineStr">
@@ -7070,11 +6090,6 @@
           <t>578</t>
         </is>
       </c>
-      <c r="B555" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="556">
       <c r="A556" t="inlineStr">
@@ -7082,11 +6097,6 @@
           <t>579</t>
         </is>
       </c>
-      <c r="B556" t="inlineStr">
-        <is>
-          <t>10, 12, 1A1A1A, 1A1A1A1A, 1A2, 2A2, 2B1A1, 2B1B, 2B2, 2C1A, 2C1B, 2C2, 2C3A, 2C3B1, 2C3B2, 3, 4, 5A, 5B, 5C, 6A, 6B, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="557">
       <c r="A557" t="inlineStr">
@@ -7094,11 +6104,6 @@
           <t>58</t>
         </is>
       </c>
-      <c r="B557" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A1A, 2A1B, 2A1C, 2A2, 2B1, 2B2</t>
-        </is>
-      </c>
     </row>
     <row r="558">
       <c r="A558" t="inlineStr">
@@ -7106,11 +6111,6 @@
           <t>580</t>
         </is>
       </c>
-      <c r="B558" t="inlineStr">
-        <is>
-          <t>1A1A, 1A1B, 1A2A, 1A2B, 1A2C, 1B, 2A1A, 2A1B, 2A2A, 2A2B, 2B1, 2B2, 2B3, 2C1, 2C2A, 2C2B1, 2C2B2</t>
-        </is>
-      </c>
     </row>
     <row r="559">
       <c r="A559" t="inlineStr">
@@ -7118,11 +6118,6 @@
           <t>581</t>
         </is>
       </c>
-      <c r="B559" t="inlineStr">
-        <is>
-          <t>12, 13, 17, 18A, 18B, 18C, 19, 1A1, 1A2, 1A3, 1B1A1, 1B1B, 1B1C1, 1B1C2, 1B2, 1B3, 1B4, 1C1A1, 1C1B, 1C2A, 1C2B, 1C3, 1D1A, 1D1B, 1D2, 20, 21, 23, 27, 28, 29, 2A1A1, 2A1A1A1A1B, 2A1A1A2, 2A1A1B1, 2A1A1C, 2A1A1D, 2A1A2A, 2A1A2B, 2A1A3, 2A1B, 2A1C, 2A1D, 2A1E, 30, 31, 32A1, 32B, 33, 34, 35A, 35B, 36, 37, 38, 39, 3A1A1, 3A1A1A1B, 3A1A1A2, 3A1A1B, 3A1B, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 4A, 4B, 50, 51, 52, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="560">
       <c r="A560" t="inlineStr">
@@ -7130,11 +6125,6 @@
           <t>582</t>
         </is>
       </c>
-      <c r="B560" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="561">
       <c r="A561" t="inlineStr">
@@ -7142,11 +6132,6 @@
           <t>583</t>
         </is>
       </c>
-      <c r="B561" t="inlineStr">
-        <is>
-          <t>1A1A, 1A1B, 1A2A, 1A2B, 1A3, 1A4, 1A5, 1A6, 1C1, 1C2A1A1, 1C2A1B, 1C2A2, 1C2B, 1C2C, 1C2D1B, 1C2D2A1, 1C2E, 2A1, 2A2, 2B1A, 2B1B, 2B2, 2C, 2D1, 2D2, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="562">
       <c r="A562" t="inlineStr">
@@ -7154,11 +6139,6 @@
           <t>584</t>
         </is>
       </c>
-      <c r="B562" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="563">
       <c r="A563" t="inlineStr">
@@ -7166,11 +6146,6 @@
           <t>585A</t>
         </is>
       </c>
-      <c r="B563" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2</t>
-        </is>
-      </c>
     </row>
     <row r="564">
       <c r="A564" t="inlineStr">
@@ -7178,11 +6153,6 @@
           <t>585B</t>
         </is>
       </c>
-      <c r="B564" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24A, 24B, 25, 26, 27, 28, 29, 2A, 2B, 2C, 2C1A1A, 2C1A1A2, 2C1A1B1, 2C1A2, 2C1B1, 2C1B2, 2C2, 2C3, 2C4, 2C5, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 3A10, 3A1A1, 3A1A1A1B, 3A1A1A2, 3A1A1A3, 3A1A1B, 3A1A2, 3A1B1, 3A1B2, 3A2, 3A3, 3A4, 3A5, 3A6, 3B1, 3B2, 40, 41, 42, 43, 44, 45, 46, 4A, 4B, 5, 6, 6A, 6B, 6C, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="565">
       <c r="A565" t="inlineStr">
@@ -7190,11 +6160,6 @@
           <t>586</t>
         </is>
       </c>
-      <c r="B565" t="inlineStr">
-        <is>
-          <t>11, 12, 13, 14, 15, 16, 17, 18, 19, 1A1A, 1A1B, 1A2, 1B, 1B2A, 1B2B1, 1B2B1A1, 1B2B2, 1B2C, 1C1, 1C1A, 1C2, 1C2A1, 1C2A1B, 1C2A2, 1C2B, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A1A, 2A1B, 2A2, 2A3, 2B, 30, 31, 3A1A1, 3A1B, 3A2, 3B, 4A1A, 4A1B, 5, 6, 7A, 7B1, 7B2, 7B3, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="566">
       <c r="A566" t="inlineStr">
@@ -7202,11 +6167,6 @@
           <t>587A</t>
         </is>
       </c>
-      <c r="B566" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="567">
       <c r="A567" t="inlineStr">
@@ -7214,11 +6174,6 @@
           <t>587B</t>
         </is>
       </c>
-      <c r="B567" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A, 1B, 20, 21, 22, 23, 24, 25, 26, 27A, 27B, 27C, 28A, 28B, 28C, 29, 2A1A, 2A1B, 2A2, 2B, 30, 31, 32, 33, 34, 35, 36, 37, 38A1, 38A2, 38B, 39, 3A, 3A1A, 3A2, 3B, 40, 41, 42, 43, 4A1A, 4A2, 4A31, 4B1A1A1, 4B1A2, 4B1B1, 4B1B2, 4B2, 4B3, 4C1A1, 4C1B1, 4C1B2, 4C2, 4C3, 5, 6A1, 6A2, 6A3, 6A4, 6B1A, 6B1B, 6B2, 6C1, 6C2, 6C3, 6C4, 6D, 7A1A1A, 7A2, 7A3, 7A4, 7B1A, 7B1B, 7B1C, 7B1C2, 7B2, 8, 9A1, 9A2, 9B1A, 9B1B, 9B2A, 9B2B, 9B2C, 9B2D</t>
-        </is>
-      </c>
     </row>
     <row r="568">
       <c r="A568" t="inlineStr">
@@ -7226,11 +6181,6 @@
           <t>588</t>
         </is>
       </c>
-      <c r="B568" t="inlineStr">
-        <is>
-          <t>1A1A, 1A1C, 1A2, 1C1A, 1C1B, 1C2, 2, 3A1A, 3A1B, 3A2A, 3A2B, 3A3, 3B1A, 3B1B, 3B2, 3C, 3D, 3E1, 3E2, 4A, 4B, 4C1A1, 4C1A2, 4C1B, 4C2, 5A1A, 5A1B1A1, 5A1B1A2, 5A1B2, 5A2, 5A3A, 5A3B, 5B, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="569">
       <c r="A569" t="inlineStr">
@@ -7238,11 +6188,6 @@
           <t>589</t>
         </is>
       </c>
-      <c r="B569" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="570">
       <c r="A570" t="inlineStr">
@@ -7250,11 +6195,6 @@
           <t>59</t>
         </is>
       </c>
-      <c r="B570" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="571">
       <c r="A571" t="inlineStr">
@@ -7262,11 +6202,6 @@
           <t>590</t>
         </is>
       </c>
-      <c r="B571" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B1, 10B2, 10B3A1A, 11, 12, 13A1, 13A2, 13B, 13C1, 13C2, 14A1A, 14A1B, 14A2, 15, 16, 17, 18A, 18B, 19A, 19B, 2, 20A, 20A1B, 20B, 21, 22A, 22B, 23A, 23B, 24, 25A, 25B, 25C, 25D1, 25D2, 25E1, 25E2, 26, 27A1, 27A2A, 27A2B, 27B, 28, 29, 3, 30, 31, 35, 36, 37, 38, 39, 4, 40, 5, 6, 7A1A, 7A1B1, 7A1B3, 7A1B4, 7A2, 7B, 8A, 8B1, 8B2, 8C, 8D, 9</t>
-        </is>
-      </c>
     </row>
     <row r="572">
       <c r="A572" t="inlineStr">
@@ -7274,11 +6209,6 @@
           <t>591</t>
         </is>
       </c>
-      <c r="B572" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1B, 2A1A, 2A1B, 2A2, 2A3, 2B, 3A1A1, 3A1A2, 3A1B, 3A2, 3A3A, 3A3B, 3A3C, 3A4, 3A5A, 3A5B, 3A5C, 3A5D, 3A5E, 3A5F, 3A5G, 3A6, 3A7, 3B1, 3B2, 3B3, 3B4, 3B5, 3B6, 3B7, 4A1A, 4A1B, 4A2, 4B1, 4B2, 4C1A, 4C1B, 4C1C, 4C1D, 4C2, 5A1, 5A2, 5B, 6A, 6B, 6C, 6D, 6E, 7A1, 7A2, 7A3, 7B, 7C, 7D, 7E, 8</t>
-        </is>
-      </c>
     </row>
     <row r="573">
       <c r="A573" t="inlineStr">
@@ -7286,11 +6216,6 @@
           <t>592A</t>
         </is>
       </c>
-      <c r="B573" t="inlineStr">
-        <is>
-          <t>1, 2A1A, 2A1B, 2A1C, 2A1D, 2A1E1, 2A1E2, 2A1F1, 2A1F2, 2A1G1, 2A1G2, 2A1H, 2A1J, 2A1K, 2A1LA, 2A1LB, 2A2A1A, 2A2A1B1, 2A2A1B2, 2A2A1C, 2A2A2, 2A2A3, 2A2A4, 2A2A5, 2A2B, 2B, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="574">
       <c r="A574" t="inlineStr">
@@ -7298,11 +6223,6 @@
           <t>592B</t>
         </is>
       </c>
-      <c r="B574" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1A3, 1B1, 1B2, 1C1, 1C2A, 1C2B, 1C3A1, 1C3A2, 1C3A3, 1C3A4, 1C3A5, 1C3A6, 1C3A7, 1C3B, 1C4A, 1C4B1, 1C4B2, 1C4C, 1C5, 1C6A1, 1C6B, 1C7, 2, 3, 4, 5, 6A</t>
-        </is>
-      </c>
     </row>
     <row r="575">
       <c r="A575" t="inlineStr">
@@ -7310,11 +6230,6 @@
           <t>592C</t>
         </is>
       </c>
-      <c r="B575" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="576">
       <c r="A576" t="inlineStr">
@@ -7322,11 +6237,6 @@
           <t>593</t>
         </is>
       </c>
-      <c r="B576" t="inlineStr">
-        <is>
-          <t>1A1A1, 1A1A2, 1A1B, 1A2A, 1A2B, 1A2C1A, 1A2C1C, 1A2C2, 1A2D, 1B1, 1B2, 1C1, 1C2A, 1C2B, 2A, 2B1, 2B2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="577">
       <c r="A577" t="inlineStr">
@@ -7334,11 +6244,6 @@
           <t>594</t>
         </is>
       </c>
-      <c r="B577" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A1A, 2A1B, 2A1C, 2A2, 2B1, 2B2, 2B3, 3A1A1A, 3A1B, 3A2, 3B, 4, 5, 6, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="578">
       <c r="A578" t="inlineStr">
@@ -7346,11 +6251,6 @@
           <t>595</t>
         </is>
       </c>
-      <c r="B578" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13, 14, 15, 16, 1A1A, 1A1B, 1A1C, 1A2, 1A3, 1A4, 1A5, 1B, 2A1, 2A2, 2B, 2C1A1A, 2C1A1B, 2C1B, 2C1C, 2C2, 3B1A1A, 5A1, 5A2A1, 5A2B, 5A2C, 5B1, 5B2, 6A1A1, 6A1A2B, 6A1A3, 6A1A4, 6A1B, 6A2A, 6A3, 6A4, 6A5, 6A6, 6B, 6C1A1, 6C1B1, 6C1B2, 6C1B3, 6C2, 6C3A, 6C3B, 6C4, 6C5, 6C6, 6C7, 7A1, 7A2, 7B1, 7B2, 8A, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="579">
       <c r="A579" t="inlineStr">
@@ -7358,11 +6258,6 @@
           <t>596</t>
         </is>
       </c>
-      <c r="B579" t="inlineStr">
-        <is>
-          <t>1A1A, 1A1B1, 1A1B2, 1A1C, 1A1D, 1A1E, 1A1F, 1A1G, 1A1H, 1A1I1, 1A1I2, 1A1J, 1A1K, 1A1L, 1A1M, 1A2A, 1A2B, 1A3A, 1A3B, 1B, 1B1A, 1B1B1A, 1B1B1B, 1B1B2, 1B1C1, 1B1C2A1A, 1B1C2A1A2, 1B1C2A1B, 1B1C2A1C, 1B1C2A2, 1B1C2B, 1B1C2C, 1B2, 1B3, 1B4, 2A1A, 2A1B, 2A2, 2B, 3A1A, 3A1B, 3A2, 3B1A1, 3B1A2, 3B1B1, 3B1B2, 3B2, 3C1A1A, 3C1A1B1A, 3C1A2, 3C1B, 3C1C1, 3C1C2A, 3C1C2B, 3C2, 4, 5, 6, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="580">
       <c r="A580" t="inlineStr">
@@ -7370,11 +6265,6 @@
           <t>597</t>
         </is>
       </c>
-      <c r="B580" t="inlineStr">
-        <is>
-          <t>10A1, 10A2, 10B, 11, 12A, 12B, 14, 1A, 1B1, 1B2, 2A, 2B, 3, 4, 5A, 5B1B, 5B2A1, 5B2A2, 5B2B1, 5B2C1A, 5B2C1B, 5B2C2, 5B3A1, 5B3A2, 5B3B1, 6A1, 6A2A, 6A2B, 6A3, 6B, 7A, 7B1, 7B1B2, 7B1B3, 7B2, 8A, 8B1, 8B2, 8C, 8D, 8E, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="581">
       <c r="A581" t="inlineStr">
@@ -7382,11 +6272,6 @@
           <t>598</t>
         </is>
       </c>
-      <c r="B581" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B, 11, 12, 13, 14, 15, 16, 17A, 17B, 18, 19, 20, 21, 22, 23, 24, 25A, 25B, 26, 27, 28A, 28B, 29A, 29B, 29C, 2A1A1, 2A1A2, 2A1B, 2A2, 2A3A1, 2A3B, 2A3C, 2A3D, 2A4, 2B, 2C, 30, 31A, 32, 33, 34, 35, 36, 37, 38, 39, 3A1, 3A2, 3A3, 3A4, 3B1, 3B2, 3C, 40, 41A, 41B, 41C, 41D, 42A, 42B, 42C, 42D, 43, 43A, 43B, 43C, 43D, 44, 45, 46, 48, 49, 4A, 4B, 5, 50, 51A, 51B, 6, 7, 8A, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="582">
       <c r="A582" t="inlineStr">
@@ -7394,11 +6279,6 @@
           <t>599</t>
         </is>
       </c>
-      <c r="B582" t="inlineStr">
-        <is>
-          <t>1, 10, 11A, 11B, 12A, 12B, 13, 14, 15, 16, 17, 18, 19A, 19B, 2, 20, 21, 22, 24, 25, 26, 27, 28, 29, 2A, 2B, 2C, 2D, 3, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49A, 49B, 4A, 4B, 5, 50, 51A, 51B, 52, 53A, 54, 55, 56, 57, 58, 59, 6, 60, 61A, 61B, 62, 63, 64, 65, 66, 67, 68, 69, 7, 70, 71A, 71B, 72, 73, 74, 75A1, 75A2, 75A3, 75A4, 75B, 76A, 76B1, 76B2, 77A1A, 77A2, 77B, 78, 79, 80, 81, 82, 8A, 8B, 8C, 8D, 8E, 8F, 8G, 9</t>
-        </is>
-      </c>
     </row>
     <row r="583">
       <c r="A583" t="inlineStr">
@@ -7406,11 +6286,6 @@
           <t>6</t>
         </is>
       </c>
-      <c r="B583" t="inlineStr">
-        <is>
-          <t>1A1A, 1A1B, 1A2, 1B1A, 1B1B, 1B1C, 1B2, 2A, 2B, 3, 4A, 4B, 4C, 5</t>
-        </is>
-      </c>
     </row>
     <row r="584">
       <c r="A584" t="inlineStr">
@@ -7418,11 +6293,6 @@
           <t>60</t>
         </is>
       </c>
-      <c r="B584" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3A, 3B, 3C, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="585">
       <c r="A585" t="inlineStr">
@@ -7430,11 +6300,6 @@
           <t>600</t>
         </is>
       </c>
-      <c r="B585" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A, 2B1, 2C, 3, 4, 8</t>
-        </is>
-      </c>
     </row>
     <row r="586">
       <c r="A586" t="inlineStr">
@@ -7442,11 +6307,6 @@
           <t>601</t>
         </is>
       </c>
-      <c r="B586" t="inlineStr">
-        <is>
-          <t>10, 1A1, 1A1A1B1A, 1A1A1B2, 1A1A1B3, 1A2, 1A3, 1A4, 2A1A2A1A1, 2A1A2A1B, 2A1A2A2, 2A1A2A3, 2A1A3A, 2A1A3B, 2A1A3C, 2A1B1, 2A1C1A, 2A1C2, 2A2A, 2A2B, 2B1, 2B2, 7A, 7B, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="587">
       <c r="A587" t="inlineStr">
@@ -7454,11 +6314,6 @@
           <t>602A</t>
         </is>
       </c>
-      <c r="B587" t="inlineStr">
-        <is>
-          <t>1, 10, 2, 3, 4A, 4B, 5A, 5B, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="588">
       <c r="A588" t="inlineStr">
@@ -7466,11 +6321,6 @@
           <t>602B</t>
         </is>
       </c>
-      <c r="B588" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="589">
       <c r="A589" t="inlineStr">
@@ -7478,11 +6328,6 @@
           <t>603</t>
         </is>
       </c>
-      <c r="B589" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13, 14, 15, 16, 1A1A2, 1A1B, 1A1B2, 1A1C, 1A1D, 1A1E, 1A1F, 1A2, 1B1A, 1B2A1A1, 1B2A2, 1B2B, 20, 21, 23, 26, 28, 29, 2A1A1A1, 2A1A1AC, 2A1A2, 2A1B, 2A2, 2B1A1, 2B1A1A, 2B1A1B, 2B1A2A, 2B1A2B, 2B1B, 2B2A1B1, 2B2A2, 2B4, 3, 30, 32, 33, 34, 35, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 4A1A, 4A1A1B, 4A1A1C, 4A1A2, 4A1A3, 4A1A4, 4A1A5, 4B, 4C, 4D, 4E1, 4E2, 4F, 4G, 5, 50, 51, 52, 53, 54, 55, 57, 6B, 7A1, 7A2, 7B1, 7B2, 8, 8A, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="590">
       <c r="A590" t="inlineStr">
@@ -7490,11 +6335,6 @@
           <t>604</t>
         </is>
       </c>
-      <c r="B590" t="inlineStr">
-        <is>
-          <t>10, 11, 13, 18, 19A, 19B, 1A1A, 1A2, 1B1, 1B2, 21, 22, 24, 26, 27, 2A1A1A, 2A1A1A2, 2A1A1AB, 2A1A1C, 2A1B, 2A2, 2B10A, 2B1A1B, 2B1A2, 2B2, 35, 36, 37A1, 37A2A, 37A2B, 37B, 38, 39, 3A, 3B1, 3B2, 3C1A, 3C1A1, 3C1A2A2, 3C1A2A3, 3C1A2B, 3C1A2C1, 3C1B, 3C2, 3C3, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 4A, 4B, 5, 50, 51, 52, 53, 54, 55, 56, 57, 58, 59, 6</t>
-        </is>
-      </c>
     </row>
     <row r="591">
       <c r="A591" t="inlineStr">
@@ -7502,11 +6342,6 @@
           <t>605</t>
         </is>
       </c>
-      <c r="B591" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13, 14, 15, 18A, 18B, 19, 1A1A1, 1A1B, 20, 21, 22A, 22B, 23A, 23B, 24, 25, 26, 2A1A, 2A1A1B, 2A1A1C, 2A1A2, 2A1B, 2A2, 2B, 3A, 3B, 4, 5, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="592">
       <c r="A592" t="inlineStr">
@@ -7514,11 +6349,6 @@
           <t>606</t>
         </is>
       </c>
-      <c r="B592" t="inlineStr">
-        <is>
-          <t>10, 10A, 12, 13, 14, 18, 19, 1A1A, 1A1B, 1A2, 1B, 20, 21, 22, 23, 24, 25, 2A1, 2A2, 2B, 36, 37, 38, 39, 3A1A1, 3A1A2, 3A1A3, 3A1B1, 3A1B2, 3A1B3, 3A2A, 3A2B, 3A2C, 3A4A, 3A4B, 3A4E2, 3B, 4, 40, 41, 42, 43, 44, 45, 46, 47, 5A1A1AA1, 5A1B, 5A2, 5B, 6A1, 6A1A2, 6A1B, 6A2A1A1, 6A2A2, 6A2B, 6B1A1A, 6B2, 6B3, 7A1A1, 7A2, 7B, 7C, 7D, 7F, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="593">
       <c r="A593" t="inlineStr">
@@ -7526,11 +6356,6 @@
           <t>607</t>
         </is>
       </c>
-      <c r="B593" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B1A1, 2B1A2, 2B1B, 2B1C1, 2B1C2, 2B2, 2C, 3A, 3B1, 3B2, 4, 5, 6A1, 6A2, 6B, 7</t>
-        </is>
-      </c>
     </row>
     <row r="594">
       <c r="A594" t="inlineStr">
@@ -7538,11 +6363,6 @@
           <t>608</t>
         </is>
       </c>
-      <c r="B594" t="inlineStr">
-        <is>
-          <t>1A, 1B1, 1B2, 2A, 2B</t>
-        </is>
-      </c>
     </row>
     <row r="595">
       <c r="A595" t="inlineStr">
@@ -7550,11 +6370,6 @@
           <t>609</t>
         </is>
       </c>
-      <c r="B595" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3A, 3B, 3C, 4, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="596">
       <c r="A596" t="inlineStr">
@@ -7562,11 +6377,6 @@
           <t>61</t>
         </is>
       </c>
-      <c r="B596" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="597">
       <c r="A597" t="inlineStr">
@@ -7574,11 +6384,6 @@
           <t>610</t>
         </is>
       </c>
-      <c r="B597" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3</t>
-        </is>
-      </c>
     </row>
     <row r="598">
       <c r="A598" t="inlineStr">
@@ -7586,11 +6391,6 @@
           <t>611</t>
         </is>
       </c>
-      <c r="B598" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 4</t>
-        </is>
-      </c>
     </row>
     <row r="599">
       <c r="A599" t="inlineStr">
@@ -7598,11 +6398,6 @@
           <t>612</t>
         </is>
       </c>
-      <c r="B599" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3A1A1, 3A1A2, 3A2A1, 3A2A2, 3A2B, 3B, 4A, 4B1, 4B2A, 4B2B1, 4B2B2, 4B2B3, 5</t>
-        </is>
-      </c>
     </row>
     <row r="600">
       <c r="A600" t="inlineStr">
@@ -7610,11 +6405,6 @@
           <t>613</t>
         </is>
       </c>
-      <c r="B600" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13, 15, 16, 17, 18, 19, 1A1A, 1A1A2, 1A2, 1B, 20, 21, 22, 23, 24, 25, 27, 28, 29, 2A1A1A1, 2A1A1AA, 2A1A1B, 2A1A2, 2A1A3, 2A1A4, 2A1B1, 2A1B2, 2A3, 2A4, 2A5, 2A6, 2B, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 3A1A1, 3A1B, 3A1C1, 3A1C2, 3A3A1B, 3B1A1A1, 3B1A2, 3B1B1A, 3B1B2, 3B1B3, 3B2, 3B3, 3B4, 3B5A, 3B5B, 3B6, 4A1A1, 4A1A1A1, 4A1A3, 4A1B, 4A2A, 4A2B, 4B1, 4B2, 5A1, 5A1A1A1, 5A2A, 5A2B, 5B, 6A1, 6B1, 7A1A1, 7A1B, 7A2, 7B1, 7B2, 7B3, 7C, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="601">
       <c r="A601" t="inlineStr">
@@ -7622,11 +6412,6 @@
           <t>614</t>
         </is>
       </c>
-      <c r="B601" t="inlineStr">
-        <is>
-          <t>10, 11A1, 11A1B, 11A2, 11B, 13, 13A, 13B, 16, 17, 19, 1A1A, 1A1B, 1A1C, 1A2, 1B, 1C1A, 1C1B1, 1C1B1A1, 1C1B1A2B, 1C1B1A2C1, 1C1B1A3, 1C1B1B, 1C1B2, 1C1B2A, 1C1B2B1, 1C1B2B2, 1C1B2C, 1C1B3, 1C1B3A1, 1C1B3A2, 1C1B3B1, 1C1B3C, 1C1B3D, 1C1B3E, 1C1B4B, 1C1B5A2, 1C1B5B1, 1C1C1A, 1C1C1B, 1C1C1BA2, 1C1C2A2, 1C1C2A3, 1C1C2B, 1C2, 1D1A1, 1D1B, 1D2A1A1, 1D2B, 1D3A1A, 1D3A1B, 1D3A2, 1E1A, 1E1B1A, 1E1B2, 1E1B3, 1E1C, 1E1D, 1E2, 1E3A1, 1E3A2A, 1E3A2B, 1E3B, 1E3C, 1E4, 1E5A1, 1E5A2, 2, 20, 23, 24, 25, 27, 29, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 3A, 3B, 4, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 50, 5A, 5B, 6, 7, 70, 75, 76, 77, 8A1, 8A2, 8B1A, 8B1B, 8B2</t>
-        </is>
-      </c>
     </row>
     <row r="602">
       <c r="A602" t="inlineStr">
@@ -7634,11 +6419,6 @@
           <t>615</t>
         </is>
       </c>
-      <c r="B602" t="inlineStr">
-        <is>
-          <t>1A1A, 1A1B, 1A2, 1B, 2</t>
-        </is>
-      </c>
     </row>
     <row r="603">
       <c r="A603" t="inlineStr">
@@ -7646,11 +6426,6 @@
           <t>616</t>
         </is>
       </c>
-      <c r="B603" t="inlineStr">
-        <is>
-          <t>1A1, 1A2B, 2B</t>
-        </is>
-      </c>
     </row>
     <row r="604">
       <c r="A604" t="inlineStr">
@@ -7658,11 +6433,6 @@
           <t>617</t>
         </is>
       </c>
-      <c r="B604" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4A1, 4A10, 4A11, 4A12, 4A13, 4A14, 4A15, 4A16, 4A17, 4A18, 4A19, 4A2, 4A20, 4A21, 4A3, 4A4, 4A5, 4A6, 4A7, 4A8, 4A9, 4B</t>
-        </is>
-      </c>
     </row>
     <row r="605">
       <c r="A605" t="inlineStr">
@@ -7670,11 +6440,6 @@
           <t>618</t>
         </is>
       </c>
-      <c r="B605" t="inlineStr">
-        <is>
-          <t>1A1TO1B7B, 2</t>
-        </is>
-      </c>
     </row>
     <row r="606">
       <c r="A606" t="inlineStr">
@@ -7682,11 +6447,6 @@
           <t>619A</t>
         </is>
       </c>
-      <c r="B606" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1B, 1C, 2</t>
-        </is>
-      </c>
     </row>
     <row r="607">
       <c r="A607" t="inlineStr">
@@ -7694,11 +6454,6 @@
           <t>619B</t>
         </is>
       </c>
-      <c r="B607" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="608">
       <c r="A608" t="inlineStr">
@@ -7706,11 +6461,6 @@
           <t>62</t>
         </is>
       </c>
-      <c r="B608" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="609">
       <c r="A609" t="inlineStr">
@@ -7718,11 +6468,6 @@
           <t>620</t>
         </is>
       </c>
-      <c r="B609" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="610">
       <c r="A610" t="inlineStr">
@@ -7730,11 +6475,6 @@
           <t>621A</t>
         </is>
       </c>
-      <c r="B610" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4A, 4B1, 4B2A, 4B2B, 4B2C, 5</t>
-        </is>
-      </c>
     </row>
     <row r="611">
       <c r="A611" t="inlineStr">
@@ -7742,11 +6482,6 @@
           <t>621B</t>
         </is>
       </c>
-      <c r="B611" t="inlineStr">
-        <is>
-          <t>1, 2A1, 2A2A, 2A2B, 2B1, 2B2, 2B3, 2B4, 2B5, 2C</t>
-        </is>
-      </c>
     </row>
     <row r="612">
       <c r="A612" t="inlineStr">
@@ -7754,11 +6489,6 @@
           <t>622</t>
         </is>
       </c>
-      <c r="B612" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1B, 2A1, 2A2, 2B</t>
-        </is>
-      </c>
     </row>
     <row r="613">
       <c r="A613" t="inlineStr">
@@ -7766,11 +6496,6 @@
           <t>623</t>
         </is>
       </c>
-      <c r="B613" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="614">
       <c r="A614" t="inlineStr">
@@ -7778,11 +6503,6 @@
           <t>624</t>
         </is>
       </c>
-      <c r="B614" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="615">
       <c r="A615" t="inlineStr">
@@ -7790,11 +6510,6 @@
           <t>625</t>
         </is>
       </c>
-      <c r="B615" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="616">
       <c r="A616" t="inlineStr">
@@ -7802,11 +6517,6 @@
           <t>626</t>
         </is>
       </c>
-      <c r="B616" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="617">
       <c r="A617" t="inlineStr">
@@ -7814,11 +6524,6 @@
           <t>627</t>
         </is>
       </c>
-      <c r="B617" t="inlineStr">
-        <is>
-          <t>1TO4B</t>
-        </is>
-      </c>
     </row>
     <row r="618">
       <c r="A618" t="inlineStr">
@@ -7826,11 +6531,6 @@
           <t>628</t>
         </is>
       </c>
-      <c r="B618" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="619">
       <c r="A619" t="inlineStr">
@@ -7838,11 +6538,6 @@
           <t>629</t>
         </is>
       </c>
-      <c r="B619" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="620">
       <c r="A620" t="inlineStr">
@@ -7850,11 +6545,6 @@
           <t>63</t>
         </is>
       </c>
-      <c r="B620" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="621">
       <c r="A621" t="inlineStr">
@@ -7862,11 +6552,6 @@
           <t>630</t>
         </is>
       </c>
-      <c r="B621" t="inlineStr">
-        <is>
-          <t>1TO4</t>
-        </is>
-      </c>
     </row>
     <row r="622">
       <c r="A622" t="inlineStr">
@@ -7874,11 +6559,6 @@
           <t>631</t>
         </is>
       </c>
-      <c r="B622" t="inlineStr">
-        <is>
-          <t>1TO4</t>
-        </is>
-      </c>
     </row>
     <row r="623">
       <c r="A623" t="inlineStr">
@@ -7886,11 +6566,6 @@
           <t>632</t>
         </is>
       </c>
-      <c r="B623" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3A, 3B, 4A, 4B</t>
-        </is>
-      </c>
     </row>
     <row r="624">
       <c r="A624" t="inlineStr">
@@ -7898,11 +6573,6 @@
           <t>633</t>
         </is>
       </c>
-      <c r="B624" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="625">
       <c r="A625" t="inlineStr">
@@ -7910,11 +6580,6 @@
           <t>634</t>
         </is>
       </c>
-      <c r="B625" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B1, 2B2, 2C1, 2C2A, 2C2B</t>
-        </is>
-      </c>
     </row>
     <row r="626">
       <c r="A626" t="inlineStr">
@@ -7922,11 +6587,6 @@
           <t>635</t>
         </is>
       </c>
-      <c r="B626" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B1TO2B5</t>
-        </is>
-      </c>
     </row>
     <row r="627">
       <c r="A627" t="inlineStr">
@@ -7934,11 +6594,6 @@
           <t>636</t>
         </is>
       </c>
-      <c r="B627" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2</t>
-        </is>
-      </c>
     </row>
     <row r="628">
       <c r="A628" t="inlineStr">
@@ -7946,11 +6601,6 @@
           <t>637</t>
         </is>
       </c>
-      <c r="B628" t="inlineStr">
-        <is>
-          <t>1A1, 1B, 2A1A, 2A1B, 2A1CTO2B, 2A3B, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="629">
       <c r="A629" t="inlineStr">
@@ -7958,11 +6608,6 @@
           <t>638</t>
         </is>
       </c>
-      <c r="B629" t="inlineStr">
-        <is>
-          <t>10A, 10B, 1A1, 1A2, 1B, 2A, 2B, 3A, 3B, 4A, 4B, 5A, 5B, 6A, 6B, 6C, 7, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="630">
       <c r="A630" t="inlineStr">
@@ -7970,11 +6615,6 @@
           <t>639</t>
         </is>
       </c>
-      <c r="B630" t="inlineStr">
-        <is>
-          <t>1, 10A, 11A, 2A, 2B, 3A1, 3A2, 3B, 4B</t>
-        </is>
-      </c>
     </row>
     <row r="631">
       <c r="A631" t="inlineStr">
@@ -7982,11 +6622,6 @@
           <t>64</t>
         </is>
       </c>
-      <c r="B631" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 2</t>
-        </is>
-      </c>
     </row>
     <row r="632">
       <c r="A632" t="inlineStr">
@@ -7994,11 +6629,6 @@
           <t>640</t>
         </is>
       </c>
-      <c r="B632" t="inlineStr">
-        <is>
-          <t>1ATO3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="633">
       <c r="A633" t="inlineStr">
@@ -8006,11 +6636,6 @@
           <t>641</t>
         </is>
       </c>
-      <c r="B633" t="inlineStr">
-        <is>
-          <t>1TO2ATO2D</t>
-        </is>
-      </c>
     </row>
     <row r="634">
       <c r="A634" t="inlineStr">
@@ -8018,11 +6643,6 @@
           <t>642</t>
         </is>
       </c>
-      <c r="B634" t="inlineStr">
-        <is>
-          <t>1ATO1C2A, 2, 3, 3A1TO3D2</t>
-        </is>
-      </c>
     </row>
     <row r="635">
       <c r="A635" t="inlineStr">
@@ -8030,11 +6650,6 @@
           <t>643</t>
         </is>
       </c>
-      <c r="B635" t="inlineStr">
-        <is>
-          <t>1A1A1A, 1A1A2A, 1A1B2, 1A2B, 1B, 2ATO2C, 3, 4, 5A, 6, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="636">
       <c r="A636" t="inlineStr">
@@ -8042,11 +6657,6 @@
           <t>644</t>
         </is>
       </c>
-      <c r="B636" t="inlineStr">
-        <is>
-          <t>1ATO1C2A, 2, 4</t>
-        </is>
-      </c>
     </row>
     <row r="637">
       <c r="A637" t="inlineStr">
@@ -8054,11 +6664,6 @@
           <t>645</t>
         </is>
       </c>
-      <c r="B637" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
     </row>
     <row r="638">
       <c r="A638" t="inlineStr">
@@ -8066,11 +6671,6 @@
           <t>646</t>
         </is>
       </c>
-      <c r="B638" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="639">
       <c r="A639" t="inlineStr">
@@ -8078,11 +6678,6 @@
           <t>647</t>
         </is>
       </c>
-      <c r="B639" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="640">
       <c r="A640" t="inlineStr">
@@ -8090,11 +6685,6 @@
           <t>648</t>
         </is>
       </c>
-      <c r="B640" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="641">
       <c r="A641" t="inlineStr">
@@ -8102,11 +6692,6 @@
           <t>649</t>
         </is>
       </c>
-      <c r="B641" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="642">
       <c r="A642" t="inlineStr">
@@ -8114,11 +6699,6 @@
           <t>65</t>
         </is>
       </c>
-      <c r="B642" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A, 2B, 2C, 3</t>
-        </is>
-      </c>
     </row>
     <row r="643">
       <c r="A643" t="inlineStr">
@@ -8126,11 +6706,6 @@
           <t>650</t>
         </is>
       </c>
-      <c r="B643" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="644">
       <c r="A644" t="inlineStr">
@@ -8138,11 +6713,6 @@
           <t>651</t>
         </is>
       </c>
-      <c r="B644" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="645">
       <c r="A645" t="inlineStr">
@@ -8150,11 +6720,6 @@
           <t>652</t>
         </is>
       </c>
-      <c r="B645" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="646">
       <c r="A646" t="inlineStr">
@@ -8162,11 +6727,6 @@
           <t>653</t>
         </is>
       </c>
-      <c r="B646" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="647">
       <c r="A647" t="inlineStr">
@@ -8174,11 +6734,6 @@
           <t>654</t>
         </is>
       </c>
-      <c r="B647" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="648">
       <c r="A648" t="inlineStr">
@@ -8186,11 +6741,6 @@
           <t>655</t>
         </is>
       </c>
-      <c r="B648" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="649">
       <c r="A649" t="inlineStr">
@@ -8198,11 +6748,6 @@
           <t>656</t>
         </is>
       </c>
-      <c r="B649" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="650">
       <c r="A650" t="inlineStr">
@@ -8210,11 +6755,6 @@
           <t>657</t>
         </is>
       </c>
-      <c r="B650" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="651">
       <c r="A651" t="inlineStr">
@@ -8222,11 +6762,6 @@
           <t>658</t>
         </is>
       </c>
-      <c r="B651" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="652">
       <c r="A652" t="inlineStr">
@@ -8234,11 +6769,6 @@
           <t>659</t>
         </is>
       </c>
-      <c r="B652" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="653">
       <c r="A653" t="inlineStr">
@@ -8246,11 +6776,6 @@
           <t>66</t>
         </is>
       </c>
-      <c r="B653" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="654">
       <c r="A654" t="inlineStr">
@@ -8258,11 +6783,6 @@
           <t>660</t>
         </is>
       </c>
-      <c r="B654" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="655">
       <c r="A655" t="inlineStr">
@@ -8270,11 +6790,6 @@
           <t>661</t>
         </is>
       </c>
-      <c r="B655" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="656">
       <c r="A656" t="inlineStr">
@@ -8282,11 +6797,6 @@
           <t>662</t>
         </is>
       </c>
-      <c r="B656" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="657">
       <c r="A657" t="inlineStr">
@@ -8294,11 +6804,6 @@
           <t>67</t>
         </is>
       </c>
-      <c r="B657" t="inlineStr">
-        <is>
-          <t>1, 2A1, 2A2, 2B</t>
-        </is>
-      </c>
     </row>
     <row r="658">
       <c r="A658" t="inlineStr">
@@ -8306,11 +6811,6 @@
           <t>68</t>
         </is>
       </c>
-      <c r="B658" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 2, 3A, 3B</t>
-        </is>
-      </c>
     </row>
     <row r="659">
       <c r="A659" t="inlineStr">
@@ -8318,11 +6818,6 @@
           <t>69</t>
         </is>
       </c>
-      <c r="B659" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="660">
       <c r="A660" t="inlineStr">
@@ -8330,11 +6825,6 @@
           <t>7</t>
         </is>
       </c>
-      <c r="B660" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 3C, 4A, 4B, 4C, 5</t>
-        </is>
-      </c>
     </row>
     <row r="661">
       <c r="A661" t="inlineStr">
@@ -8342,11 +6832,6 @@
           <t>70</t>
         </is>
       </c>
-      <c r="B661" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3A, 3B, 4</t>
-        </is>
-      </c>
     </row>
     <row r="662">
       <c r="A662" t="inlineStr">
@@ -8354,11 +6839,6 @@
           <t>71</t>
         </is>
       </c>
-      <c r="B662" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 2</t>
-        </is>
-      </c>
     </row>
     <row r="663">
       <c r="A663" t="inlineStr">
@@ -8366,11 +6846,6 @@
           <t>72</t>
         </is>
       </c>
-      <c r="B663" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="664">
       <c r="A664" t="inlineStr">
@@ -8378,11 +6853,6 @@
           <t>73</t>
         </is>
       </c>
-      <c r="B664" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="665">
       <c r="A665" t="inlineStr">
@@ -8390,11 +6860,6 @@
           <t>74</t>
         </is>
       </c>
-      <c r="B665" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="666">
       <c r="A666" t="inlineStr">
@@ -8402,11 +6867,6 @@
           <t>75</t>
         </is>
       </c>
-      <c r="B666" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3, 4, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="667">
       <c r="A667" t="inlineStr">
@@ -8414,11 +6874,6 @@
           <t>76</t>
         </is>
       </c>
-      <c r="B667" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A, 2B</t>
-        </is>
-      </c>
     </row>
     <row r="668">
       <c r="A668" t="inlineStr">
@@ -8426,11 +6881,6 @@
           <t>77</t>
         </is>
       </c>
-      <c r="B668" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B</t>
-        </is>
-      </c>
     </row>
     <row r="669">
       <c r="A669" t="inlineStr">
@@ -8438,11 +6888,6 @@
           <t>78</t>
         </is>
       </c>
-      <c r="B669" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="670">
       <c r="A670" t="inlineStr">
@@ -8450,11 +6895,6 @@
           <t>79</t>
         </is>
       </c>
-      <c r="B670" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3A, 3B, 4</t>
-        </is>
-      </c>
     </row>
     <row r="671">
       <c r="A671" t="inlineStr">
@@ -8462,11 +6902,6 @@
           <t>8</t>
         </is>
       </c>
-      <c r="B671" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 2A, 2B, 2C</t>
-        </is>
-      </c>
     </row>
     <row r="672">
       <c r="A672" t="inlineStr">
@@ -8474,11 +6909,6 @@
           <t>80</t>
         </is>
       </c>
-      <c r="B672" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="673">
       <c r="A673" t="inlineStr">
@@ -8486,11 +6916,6 @@
           <t>81</t>
         </is>
       </c>
-      <c r="B673" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="674">
       <c r="A674" t="inlineStr">
@@ -8498,11 +6923,6 @@
           <t>82</t>
         </is>
       </c>
-      <c r="B674" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="675">
       <c r="A675" t="inlineStr">
@@ -8510,11 +6930,6 @@
           <t>83</t>
         </is>
       </c>
-      <c r="B675" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="676">
       <c r="A676" t="inlineStr">
@@ -8522,11 +6937,6 @@
           <t>84</t>
         </is>
       </c>
-      <c r="B676" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="677">
       <c r="A677" t="inlineStr">
@@ -8534,11 +6944,6 @@
           <t>85</t>
         </is>
       </c>
-      <c r="B677" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4A, 4B</t>
-        </is>
-      </c>
     </row>
     <row r="678">
       <c r="A678" t="inlineStr">
@@ -8546,11 +6951,6 @@
           <t>86</t>
         </is>
       </c>
-      <c r="B678" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="679">
       <c r="A679" t="inlineStr">
@@ -8558,11 +6958,6 @@
           <t>87</t>
         </is>
       </c>
-      <c r="B679" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="680">
       <c r="A680" t="inlineStr">
@@ -8570,11 +6965,6 @@
           <t>88</t>
         </is>
       </c>
-      <c r="B680" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="681">
       <c r="A681" t="inlineStr">
@@ -8582,11 +6972,6 @@
           <t>89</t>
         </is>
       </c>
-      <c r="B681" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="682">
       <c r="A682" t="inlineStr">
@@ -8594,11 +6979,6 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B682" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="683">
       <c r="A683" t="inlineStr">
@@ -8606,11 +6986,6 @@
           <t>90</t>
         </is>
       </c>
-      <c r="B683" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3, 4, 5, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="684">
       <c r="A684" t="inlineStr">
@@ -8618,11 +6993,6 @@
           <t>91</t>
         </is>
       </c>
-      <c r="B684" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B1, 2B2</t>
-        </is>
-      </c>
     </row>
     <row r="685">
       <c r="A685" t="inlineStr">
@@ -8630,11 +7000,6 @@
           <t>92</t>
         </is>
       </c>
-      <c r="B685" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 2C, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="686">
       <c r="A686" t="inlineStr">
@@ -8642,11 +7007,6 @@
           <t>93</t>
         </is>
       </c>
-      <c r="B686" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1B1, 1B2, 2</t>
-        </is>
-      </c>
     </row>
     <row r="687">
       <c r="A687" t="inlineStr">
@@ -8654,11 +7014,6 @@
           <t>94</t>
         </is>
       </c>
-      <c r="B687" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="688">
       <c r="A688" t="inlineStr">
@@ -8666,11 +7021,6 @@
           <t>95</t>
         </is>
       </c>
-      <c r="B688" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1B, 1C, 1D, 2A1, 2A2, 2B1, 2B2</t>
-        </is>
-      </c>
     </row>
     <row r="689">
       <c r="A689" t="inlineStr">
@@ -8678,11 +7028,6 @@
           <t>96</t>
         </is>
       </c>
-      <c r="B689" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="690">
       <c r="A690" t="inlineStr">
@@ -8690,11 +7035,6 @@
           <t>97</t>
         </is>
       </c>
-      <c r="B690" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="691">
       <c r="A691" t="inlineStr">
@@ -8702,21 +7042,11 @@
           <t>98</t>
         </is>
       </c>
-      <c r="B691" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="692">
       <c r="A692" t="inlineStr">
         <is>
           <t>99</t>
-        </is>
-      </c>
-      <c r="B692" t="inlineStr">
-        <is>
-          <t>1, 2A1, 2A2, 2B, 2C, 2D</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 23 village workbooks (randomwalk-TRX50-WS 2026-10-09T11:30:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Old_Gummidipoondi_13.406625_80.12876.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Old_Gummidipoondi_13.406625_80.12876.xlsx
@@ -4718,6 +4718,11 @@
           <t>41</t>
         </is>
       </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C, 4A, 4B, 4C, 5A, 5B, 5C</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -4725,6 +4730,11 @@
           <t>410</t>
         </is>
       </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -4732,6 +4742,11 @@
           <t>411</t>
         </is>
       </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -4739,6 +4754,11 @@
           <t>412</t>
         </is>
       </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1A, 1B1B, 1B1C, 1B1D, 1B2, 2A1, 2A2, 2B, 3A1, 3A2, 3B, 4A, 4B, 4C1A1, 4C1A2, 4C1B1, 4C1B2, 4C2A, 4C2B1A1, 4C2B1A2, 4C2B1A3, 4C2B1A4, 4C2B1B, 4C2B2, 4C2B3A, 4C2B3B, 4C2B4A, 4C2B4B, 4C2B5A, 4C2B5B, 4C3A1, 4C3A2, 4C3B</t>
+        </is>
+      </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -4746,6 +4766,11 @@
           <t>413</t>
         </is>
       </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -4753,6 +4778,11 @@
           <t>414</t>
         </is>
       </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>10, 11A, 11B, 12, 13, 14, 15A, 15B1, 15B2, 15C, 16, 17A, 17B, 17C, 18, 19, 1A1, 1A2A, 1A2B1, 1B1A, 1B1B, 1B2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A1, 2A2, 2A3, 2A4, 2A5, 2A6A, 2A6B, 2A7, 2A8, 2B1, 2B2, 2B3, 2B4, 2B5, 2B6, 2B7, 2B8, 3A, 3B, 3C1A, 3C1B, 3C2, 4, 5A1A, 5A1B, 5A1C, 5A1D, 5A2, 5B, 6A1, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -4760,6 +4790,11 @@
           <t>415</t>
         </is>
       </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1A, 1B1B, 1B2, 1B3A, 1B3B, 1B3C, 1B4, 1B5, 1B6A1, 1B6A2A, 1B6A2B, 1B6B, 1B7A, 1B7B, 1C, 2A, 2B, 3A, 3B1, 3B2, 4A, 4B, 4C, 4D, 4E, 4F1, 4F2</t>
+        </is>
+      </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -4767,6 +4802,11 @@
           <t>416</t>
         </is>
       </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 4C</t>
+        </is>
+      </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -4774,6 +4814,11 @@
           <t>417</t>
         </is>
       </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 5C, 6</t>
+        </is>
+      </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -4781,6 +4826,11 @@
           <t>418</t>
         </is>
       </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B1A, 1B1B, 1B2A, 1B2B, 1B2C, 1B3, 1B4A, 1B4B, 1B4C, 1B5A, 1B5B, 2A, 2B, 2C, 2D1, 2D2, 2E1, 2E2, 2F, 2G1, 2G2, 2G3, 2H1, 2H2, 2I, 2J</t>
+        </is>
+      </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -4788,6 +4838,11 @@
           <t>419</t>
         </is>
       </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>1A, 1B10, 1B11A1, 1B11B, 1B11C, 1B11D, 1B1A, 1B1B, 1B1C, 1B2A, 1B2B, 1B3A1, 1B3A2, 1B3B, 1B3C, 1B4, 1B5, 1B6, 1B7A, 1B7B, 1B7C, 1B7D, 1B8A, 1B8B, 1B9, 1C, 2A1, 2A2, 2B, 2C, 3A1, 3A2, 3B, 4A1, 4A2, 4B1, 4B2, 4C, 4D</t>
+        </is>
+      </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
@@ -4795,6 +4850,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
@@ -4802,6 +4862,11 @@
           <t>420</t>
         </is>
       </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1B3, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
@@ -4809,6 +4874,11 @@
           <t>421</t>
         </is>
       </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3A, 3B, 3C, 4, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
@@ -4816,6 +4886,11 @@
           <t>422</t>
         </is>
       </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2A, 2B, 2C, 3A, 3B, 3C, 3D, 4A, 4B, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
@@ -4823,6 +4898,11 @@
           <t>423</t>
         </is>
       </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
@@ -4830,6 +4910,11 @@
           <t>424</t>
         </is>
       </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B1, 1B2, 2A, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
@@ -4837,6 +4922,11 @@
           <t>425</t>
         </is>
       </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
@@ -4844,6 +4934,11 @@
           <t>426</t>
         </is>
       </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
@@ -4851,6 +4946,11 @@
           <t>427</t>
         </is>
       </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
@@ -4858,6 +4958,11 @@
           <t>428</t>
         </is>
       </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
@@ -4865,6 +4970,11 @@
           <t>429</t>
         </is>
       </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
@@ -4872,6 +4982,11 @@
           <t>43</t>
         </is>
       </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
@@ -4879,6 +4994,11 @@
           <t>430</t>
         </is>
       </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
@@ -4886,6 +5006,11 @@
           <t>431</t>
         </is>
       </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
@@ -4893,6 +5018,11 @@
           <t>432</t>
         </is>
       </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
@@ -4900,6 +5030,11 @@
           <t>433</t>
         </is>
       </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
@@ -4907,6 +5042,11 @@
           <t>434</t>
         </is>
       </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
@@ -4914,6 +5054,11 @@
           <t>435</t>
         </is>
       </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
@@ -4921,6 +5066,11 @@
           <t>436</t>
         </is>
       </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1A4, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
@@ -4928,6 +5078,11 @@
           <t>437</t>
         </is>
       </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
@@ -4935,6 +5090,11 @@
           <t>438</t>
         </is>
       </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
@@ -4942,6 +5102,11 @@
           <t>439</t>
         </is>
       </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
@@ -4949,6 +5114,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
@@ -4956,6 +5126,11 @@
           <t>440</t>
         </is>
       </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
@@ -4963,6 +5138,11 @@
           <t>441</t>
         </is>
       </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C1A, 3C1B, 3C2, 3D, 3E1, 3E2</t>
+        </is>
+      </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
@@ -4970,6 +5150,11 @@
           <t>442</t>
         </is>
       </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
@@ -4977,6 +5162,11 @@
           <t>443</t>
         </is>
       </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
@@ -4984,6 +5174,11 @@
           <t>444</t>
         </is>
       </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>1A1, 1A2A, 1A2B, 1B, 2, 3, 4A, 4B, 4C, 5A1, 5A2, 5A3, 5B1, 5B2, 6A1A, 6A2, 6A3, 6A4, 6B, 7, 8A1, 8A2A1, 8A2A2, 8A2B, 8A2C, 8B1A, 8B1B, 8B2</t>
+        </is>
+      </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
@@ -4991,6 +5186,11 @@
           <t>445</t>
         </is>
       </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
@@ -4998,6 +5198,11 @@
           <t>446</t>
         </is>
       </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B, 3A, 3B, 3C</t>
+        </is>
+      </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
@@ -5005,6 +5210,11 @@
           <t>447</t>
         </is>
       </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16A, 16B, 17A, 17B, 18A, 18B, 19, 1A, 1B, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A, 2B, 3, 30, 31, 32, 33A, 33B, 34, 35A, 35B, 36, 37, 38, 39, 4, 40, 41, 42A, 42B, 5, 6, 7A, 7B, 8A, 8B, 8C, 9</t>
+        </is>
+      </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
@@ -5012,6 +5222,11 @@
           <t>448</t>
         </is>
       </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
@@ -5019,6 +5234,11 @@
           <t>449</t>
         </is>
       </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
@@ -5026,6 +5246,11 @@
           <t>45</t>
         </is>
       </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
@@ -5033,6 +5258,11 @@
           <t>450</t>
         </is>
       </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
@@ -5040,6 +5270,11 @@
           <t>451</t>
         </is>
       </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1C, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
@@ -5047,6 +5282,11 @@
           <t>452</t>
         </is>
       </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
@@ -5054,6 +5294,11 @@
           <t>453</t>
         </is>
       </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
@@ -5061,6 +5306,11 @@
           <t>454</t>
         </is>
       </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B, 1C, 1D, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
@@ -5068,6 +5318,11 @@
           <t>455</t>
         </is>
       </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>10, 1A1A1A1A, 1A1A2, 1A1A3, 1A1B, 1A2, 1A3, 1B, 2A, 2B, 2C, 3A1, 3A2A, 3A2B, 3B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
@@ -5075,6 +5330,11 @@
           <t>456</t>
         </is>
       </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
@@ -5082,6 +5342,11 @@
           <t>457</t>
         </is>
       </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>10, 11, 1A1A, 1A2, 1A3, 1B, 2A, 2B, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
@@ -5089,6 +5354,11 @@
           <t>458</t>
         </is>
       </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
@@ -5096,11 +5366,21 @@
           <t>459</t>
         </is>
       </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
           <t>46</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 24 village workbooks (rw-rtx-3070 2026-10-09T14:20:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Old_Gummidipoondi_13.406625_80.12876.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Old_Gummidipoondi_13.406625_80.12876.xlsx
@@ -4922,6 +4922,11 @@
           <t>425</t>
         </is>
       </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
@@ -4929,6 +4934,11 @@
           <t>426</t>
         </is>
       </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
@@ -4936,6 +4946,11 @@
           <t>427</t>
         </is>
       </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
@@ -4943,6 +4958,11 @@
           <t>428</t>
         </is>
       </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
@@ -4950,6 +4970,11 @@
           <t>429</t>
         </is>
       </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
@@ -4957,6 +4982,11 @@
           <t>43</t>
         </is>
       </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
@@ -4964,6 +4994,11 @@
           <t>430</t>
         </is>
       </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
@@ -4971,6 +5006,11 @@
           <t>431</t>
         </is>
       </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
@@ -4978,6 +5018,11 @@
           <t>432</t>
         </is>
       </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
@@ -4985,6 +5030,11 @@
           <t>433</t>
         </is>
       </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
@@ -4992,6 +5042,11 @@
           <t>434</t>
         </is>
       </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
@@ -4999,6 +5054,11 @@
           <t>435</t>
         </is>
       </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
@@ -5006,6 +5066,11 @@
           <t>436</t>
         </is>
       </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1A4, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
@@ -5013,6 +5078,11 @@
           <t>437</t>
         </is>
       </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
@@ -5020,6 +5090,11 @@
           <t>438</t>
         </is>
       </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
@@ -5027,6 +5102,11 @@
           <t>439</t>
         </is>
       </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
@@ -5034,6 +5114,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
@@ -5041,6 +5126,11 @@
           <t>440</t>
         </is>
       </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
@@ -5048,6 +5138,11 @@
           <t>441</t>
         </is>
       </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C1A, 3C1B, 3C2, 3D, 3E1, 3E2</t>
+        </is>
+      </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
@@ -5055,6 +5150,11 @@
           <t>442</t>
         </is>
       </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
@@ -5062,6 +5162,11 @@
           <t>443</t>
         </is>
       </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
@@ -5069,6 +5174,11 @@
           <t>444</t>
         </is>
       </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>1A1, 1A2A, 1A2B, 1B, 2, 3, 4A, 4B, 4C, 5A1, 5A2, 5A3, 5B1, 5B2, 6A1A, 6A2, 6A3, 6A4, 6B, 7, 8A1, 8A2A1, 8A2A2, 8A2B, 8A2C, 8B1A, 8B1B, 8B2</t>
+        </is>
+      </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
@@ -5076,6 +5186,11 @@
           <t>445</t>
         </is>
       </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
@@ -5083,6 +5198,11 @@
           <t>446</t>
         </is>
       </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B, 3A, 3B, 3C</t>
+        </is>
+      </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
@@ -5090,6 +5210,11 @@
           <t>447</t>
         </is>
       </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16A, 16B, 17A, 17B, 18A, 18B, 19, 1A, 1B, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A, 2B, 3, 30, 31, 32, 33A, 33B, 34, 35A, 35B, 36, 37, 38, 39, 4, 40, 41, 42A, 42B, 5, 6, 7A, 7B, 8A, 8B, 8C, 9</t>
+        </is>
+      </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
@@ -5097,6 +5222,11 @@
           <t>448</t>
         </is>
       </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
@@ -5104,6 +5234,11 @@
           <t>449</t>
         </is>
       </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
@@ -5111,6 +5246,11 @@
           <t>45</t>
         </is>
       </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
@@ -5118,6 +5258,11 @@
           <t>450</t>
         </is>
       </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
@@ -5125,6 +5270,11 @@
           <t>451</t>
         </is>
       </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1C, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
@@ -5132,6 +5282,11 @@
           <t>452</t>
         </is>
       </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
@@ -5139,6 +5294,11 @@
           <t>453</t>
         </is>
       </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
@@ -5146,6 +5306,11 @@
           <t>454</t>
         </is>
       </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B, 1C, 1D, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
@@ -5153,6 +5318,11 @@
           <t>455</t>
         </is>
       </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>10, 1A1A1A1A, 1A1A2, 1A1A3, 1A1B, 1A2, 1A3, 1B, 2A, 2B, 2C, 3A1, 3A2A, 3A2B, 3B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
@@ -5160,6 +5330,11 @@
           <t>456</t>
         </is>
       </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
@@ -5167,6 +5342,11 @@
           <t>457</t>
         </is>
       </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>10, 11, 1A1A, 1A2, 1A3, 1B, 2A, 2B, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
@@ -5174,6 +5354,11 @@
           <t>458</t>
         </is>
       </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
@@ -5181,6 +5366,11 @@
           <t>459</t>
         </is>
       </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
@@ -5188,6 +5378,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
@@ -5195,6 +5390,11 @@
           <t>460</t>
         </is>
       </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 1C, 2A1, 2A2, 2B, 3A1, 3B, 3C, 4A, 4B, 5, 6, 7A, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
@@ -5202,6 +5402,11 @@
           <t>461</t>
         </is>
       </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
@@ -5209,6 +5414,11 @@
           <t>462</t>
         </is>
       </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2, 2B1, 2B2, 2C, 2D, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
@@ -5216,6 +5426,11 @@
           <t>463</t>
         </is>
       </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
@@ -5223,6 +5438,11 @@
           <t>464</t>
         </is>
       </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1A1, 2A1A2, 2A1A3, 2A1A4, 2A1B, 2A1C, 2A2A, 2A2B, 2A2C, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
@@ -5230,6 +5450,11 @@
           <t>465</t>
         </is>
       </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C1, 2C2A, 2C2B</t>
+        </is>
+      </c>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
@@ -5237,6 +5462,11 @@
           <t>466</t>
         </is>
       </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
@@ -5244,6 +5474,11 @@
           <t>467</t>
         </is>
       </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
@@ -5251,6 +5486,11 @@
           <t>468</t>
         </is>
       </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>1A, 1B1A, 1B1B, 1B2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
@@ -5258,6 +5498,11 @@
           <t>469</t>
         </is>
       </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1A4, 1A5, 1A6, 1A7, 1A8, 1B, 2A1, 2A2, 2A3, 2A4, 2B1, 2B2, 2B3, 2B4A, 2B4B, 2C, 2D1, 2D2, 2D3, 3A, 3B, 4A, 4B1, 4B2A1A, 4B2A2, 4B2B, 4B3, 5A1A1, 5A2, 5A3, 5B, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
@@ -5265,6 +5510,11 @@
           <t>47</t>
         </is>
       </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="426">
       <c r="A426" t="inlineStr">
@@ -5272,6 +5522,11 @@
           <t>470</t>
         </is>
       </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
@@ -5279,6 +5534,11 @@
           <t>471</t>
         </is>
       </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
@@ -5286,6 +5546,11 @@
           <t>472</t>
         </is>
       </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
@@ -5293,6 +5558,11 @@
           <t>473</t>
         </is>
       </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
@@ -5300,6 +5570,11 @@
           <t>474</t>
         </is>
       </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>1, 10, 100, 101, 102, 103, 104, 105, 106, 107, 108, 109, 11, 110, 111, 112, 113, 114, 115, 116, 117, 118, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 3, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 4, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 5, 50, 51, 52, 53, 54, 55, 56, 57, 58, 59, 6, 60, 61, 62, 63, 64, 65, 66, 67, 68, 69, 70, 71, 72, 73, 74, 75, 76, 77, 78, 79, 7A, 7B, 8, 80, 81, 82, 83, 84, 85, 86, 87, 88, 89, 9, 90, 91, 92, 93, 94, 95, 96, 97, 98, 99</t>
+        </is>
+      </c>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
@@ -5307,6 +5582,11 @@
           <t>475</t>
         </is>
       </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>1, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A1, 2A2, 2A3, 2B1, 2B10, 2B11, 2B12, 2B13, 2B14, 2B15, 2B16, 2B17A, 2B17B, 2B18A, 2B18B, 2B18C, 2B19, 2B2, 2B3, 2B4, 2B5, 2B6, 2B7, 2B8, 2B9, 2C1A1, 2C1B, 2C2A1, 2C2A2, 2C2B, 2C3, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 50, 51, 52, 53, 54, 55, 56, 57, 58, 59, 60, 61, 62, 63, 64, 65, 66, 67, 68, 69, 70, 71, 72, 73, 74, 75, 76, 77, 78, 79, 80, 81, 82, 83, 84, 85, 86</t>
+        </is>
+      </c>
     </row>
     <row r="432">
       <c r="A432" t="inlineStr">
@@ -5314,6 +5594,11 @@
           <t>476</t>
         </is>
       </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="433">
       <c r="A433" t="inlineStr">
@@ -5321,6 +5606,11 @@
           <t>477</t>
         </is>
       </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
@@ -5328,6 +5618,11 @@
           <t>478</t>
         </is>
       </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
@@ -5335,6 +5630,11 @@
           <t>479</t>
         </is>
       </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>1, 21, 2A1, 2A2, 2B1A1A, 2B1A1B, 2B1A2A, 2B1A2B, 2B1A2C, 2B1A2D, 2B1A2E, 2B1B, 2B2, 4A, 4B, 4C, 4D, 5B1, 5B2, 5B3, 5B4, 6, 7A1A1, 7A1A2A, 7A1A2B, 7A1B, 7A2, 7A2A1, 7A2A2, 7A2A3, 7A2A4, 7A2B1, 7A2B10, 7A2B12, 7A2B13, 7A2B14, 7A2B15A1, 7A2B2A, 7A2B2B, 7A2B3, 7A2B4, 7A2B5, 7A2B6, 7A2B7A, 7A2B7B, 7A2B8A, 7A2B8B, 7A2B9, 7B1A, 7B1B, 7B2A, 7B2B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="436">
       <c r="A436" t="inlineStr">
@@ -5342,6 +5642,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
@@ -5349,6 +5654,11 @@
           <t>480</t>
         </is>
       </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
@@ -5356,6 +5666,11 @@
           <t>481</t>
         </is>
       </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="439">
       <c r="A439" t="inlineStr">
@@ -5363,6 +5678,11 @@
           <t>482</t>
         </is>
       </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
@@ -5370,6 +5690,11 @@
           <t>483</t>
         </is>
       </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 19, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A, 2B, 2C, 30, 31, 3A1A1, 3A1B, 3A2, 3B, 4A, 4B1, 4B2A1A, 5A1, 5A1B, 5A1C1A, 5A1C2, 5A2, 5B1A, 5B1B, 5B1C, 5B2, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="441">
       <c r="A441" t="inlineStr">
@@ -5377,6 +5702,11 @@
           <t>484</t>
         </is>
       </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
@@ -5384,6 +5714,11 @@
           <t>485</t>
         </is>
       </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>1, 1A1, 1A2A, 1A2B, 1A2C, 1A3, 1B1, 1B2, 1B3, 1C1, 1C2A, 1C2B, 1C2C, 1D1, 1D2A1, 1D2A2, 1D2B, 1D2C, 1D2D, 1D2E, 1E1, 1E2A, 1E2B, 1E2C, 1E3, 1F, 2</t>
+        </is>
+      </c>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
@@ -5391,6 +5726,11 @@
           <t>486</t>
         </is>
       </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
@@ -5398,6 +5738,11 @@
           <t>487</t>
         </is>
       </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>10, 11, 12A, 12B, 1A1A1, 1B, 1C, 1D, 1E, 1F, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
@@ -5405,6 +5750,11 @@
           <t>488</t>
         </is>
       </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
@@ -5412,6 +5762,11 @@
           <t>489</t>
         </is>
       </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>1A1, 1A2A, 1A2B1, 1A2B2, 1B, 1C1, 1C2, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="447">
       <c r="A447" t="inlineStr">
@@ -5419,6 +5774,11 @@
           <t>49</t>
         </is>
       </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 1C, 1D, 2</t>
+        </is>
+      </c>
     </row>
     <row r="448">
       <c r="A448" t="inlineStr">
@@ -5426,6 +5786,11 @@
           <t>490</t>
         </is>
       </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="449">
       <c r="A449" t="inlineStr">
@@ -5433,6 +5798,11 @@
           <t>491</t>
         </is>
       </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="450">
       <c r="A450" t="inlineStr">
@@ -5440,6 +5810,11 @@
           <t>492</t>
         </is>
       </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="451">
       <c r="A451" t="inlineStr">
@@ -5447,6 +5822,11 @@
           <t>493</t>
         </is>
       </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
@@ -5454,6 +5834,11 @@
           <t>494</t>
         </is>
       </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
@@ -5461,6 +5846,11 @@
           <t>495</t>
         </is>
       </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
@@ -5468,6 +5858,11 @@
           <t>496</t>
         </is>
       </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3A, 3B, 4, 5, 6A, 6B, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
@@ -5475,6 +5870,11 @@
           <t>497</t>
         </is>
       </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8A, 8B</t>
+        </is>
+      </c>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
@@ -5482,6 +5882,11 @@
           <t>498A</t>
         </is>
       </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="457">
       <c r="A457" t="inlineStr">
@@ -5489,6 +5894,11 @@
           <t>498B</t>
         </is>
       </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="458">
       <c r="A458" t="inlineStr">
@@ -5496,6 +5906,11 @@
           <t>499</t>
         </is>
       </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="459">
       <c r="A459" t="inlineStr">
@@ -5503,6 +5918,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
@@ -5510,6 +5930,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
@@ -5517,6 +5942,11 @@
           <t>500A</t>
         </is>
       </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="462">
       <c r="A462" t="inlineStr">
@@ -5524,6 +5954,11 @@
           <t>500B</t>
         </is>
       </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="463">
       <c r="A463" t="inlineStr">
@@ -5531,6 +5966,11 @@
           <t>501</t>
         </is>
       </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="464">
       <c r="A464" t="inlineStr">
@@ -5538,6 +5978,11 @@
           <t>502</t>
         </is>
       </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="465">
       <c r="A465" t="inlineStr">
@@ -5545,6 +5990,11 @@
           <t>503A</t>
         </is>
       </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="466">
       <c r="A466" t="inlineStr">
@@ -5552,6 +6002,11 @@
           <t>503B</t>
         </is>
       </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="467">
       <c r="A467" t="inlineStr">
@@ -5559,6 +6014,11 @@
           <t>504A</t>
         </is>
       </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="468">
       <c r="A468" t="inlineStr">
@@ -5566,6 +6026,11 @@
           <t>504B</t>
         </is>
       </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>1, 2A1A, 2A1B, 2A1C, 2A2, 2B1, 2B2, 3A1, 3A2, 3A3, 3A4, 3A5, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="469">
       <c r="A469" t="inlineStr">
@@ -5573,6 +6038,11 @@
           <t>505</t>
         </is>
       </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B1, 2B2, 2C1, 2C2</t>
+        </is>
+      </c>
     </row>
     <row r="470">
       <c r="A470" t="inlineStr">
@@ -5580,6 +6050,11 @@
           <t>506A</t>
         </is>
       </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="471">
       <c r="A471" t="inlineStr">
@@ -5587,6 +6062,11 @@
           <t>506B</t>
         </is>
       </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="472">
       <c r="A472" t="inlineStr">
@@ -5594,6 +6074,11 @@
           <t>507</t>
         </is>
       </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="473">
       <c r="A473" t="inlineStr">
@@ -5601,6 +6086,11 @@
           <t>508</t>
         </is>
       </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="474">
       <c r="A474" t="inlineStr">
@@ -5608,11 +6098,21 @@
           <t>509</t>
         </is>
       </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2A1A1A1, 2A1B, 2A2, 2A4, 2B, 2C, 3A15A1, 3A1A1, 3A1A2, 3A1B, 3A1C, 3A2, 3A3, 3A4A, 3A4B, 3A4C, 3A5A1B, 3A5A2, 3A5B, 3B, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="475">
       <c r="A475" t="inlineStr">
         <is>
           <t>51</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 25 village workbooks (rw-rtx-3070 2026-10-09T14:30:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Old_Gummidipoondi_13.406625_80.12876.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Old_Gummidipoondi_13.406625_80.12876.xlsx
@@ -6122,6 +6122,11 @@
           <t>510</t>
         </is>
       </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="477">
       <c r="A477" t="inlineStr">
@@ -6129,6 +6134,11 @@
           <t>511</t>
         </is>
       </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2A, 1A2B, 1B1A1, 1B1A2, 1B1A3, 1B1B, 1B2, 1B3, 2A, 2B1, 2B2, 3A, 3B1A1, 3B1A2A1, 3B1A2A2, 3B1B, 3B2A, 3B2B, 4A, 4B, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="478">
       <c r="A478" t="inlineStr">
@@ -6136,6 +6146,11 @@
           <t>512</t>
         </is>
       </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="479">
       <c r="A479" t="inlineStr">
@@ -6143,6 +6158,11 @@
           <t>514</t>
         </is>
       </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="480">
       <c r="A480" t="inlineStr">
@@ -6150,6 +6170,11 @@
           <t>516</t>
         </is>
       </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="481">
       <c r="A481" t="inlineStr">
@@ -6157,6 +6182,11 @@
           <t>517</t>
         </is>
       </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="482">
       <c r="A482" t="inlineStr">
@@ -6164,6 +6194,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="483">
       <c r="A483" t="inlineStr">
@@ -6171,6 +6206,11 @@
           <t>522</t>
         </is>
       </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="484">
       <c r="A484" t="inlineStr">
@@ -6178,6 +6218,11 @@
           <t>523</t>
         </is>
       </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="485">
       <c r="A485" t="inlineStr">
@@ -6185,6 +6230,11 @@
           <t>524</t>
         </is>
       </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="486">
       <c r="A486" t="inlineStr">
@@ -6192,6 +6242,11 @@
           <t>525</t>
         </is>
       </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="487">
       <c r="A487" t="inlineStr">
@@ -6199,6 +6254,11 @@
           <t>526</t>
         </is>
       </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="488">
       <c r="A488" t="inlineStr">
@@ -6206,6 +6266,11 @@
           <t>527</t>
         </is>
       </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="489">
       <c r="A489" t="inlineStr">
@@ -6213,6 +6278,11 @@
           <t>528A</t>
         </is>
       </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="490">
       <c r="A490" t="inlineStr">
@@ -6220,6 +6290,11 @@
           <t>528B</t>
         </is>
       </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="491">
       <c r="A491" t="inlineStr">
@@ -6227,6 +6302,11 @@
           <t>529A</t>
         </is>
       </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="492">
       <c r="A492" t="inlineStr">
@@ -6234,6 +6314,11 @@
           <t>529B</t>
         </is>
       </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="493">
       <c r="A493" t="inlineStr">
@@ -6241,6 +6326,11 @@
           <t>53</t>
         </is>
       </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="494">
       <c r="A494" t="inlineStr">
@@ -6248,6 +6338,11 @@
           <t>530A</t>
         </is>
       </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1A3A, 1A3B, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="495">
       <c r="A495" t="inlineStr">
@@ -6255,6 +6350,11 @@
           <t>530B</t>
         </is>
       </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="496">
       <c r="A496" t="inlineStr">
@@ -6262,6 +6362,11 @@
           <t>531</t>
         </is>
       </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2A, 2B2B, 2B2C</t>
+        </is>
+      </c>
     </row>
     <row r="497">
       <c r="A497" t="inlineStr">
@@ -6269,6 +6374,11 @@
           <t>532A</t>
         </is>
       </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B1A, 3B1B, 3B2A, 3B2B, 4, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="498">
       <c r="A498" t="inlineStr">
@@ -6276,6 +6386,11 @@
           <t>532B</t>
         </is>
       </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2A, 2A2B, 2A2C, 2A3, 2A4A, 2A4B, 2A4C, 2A4D, 2B1A, 2B1B, 2B1C, 2B2A, 2B2B, 2C1, 2C2</t>
+        </is>
+      </c>
     </row>
     <row r="499">
       <c r="A499" t="inlineStr">
@@ -6283,6 +6398,11 @@
           <t>533</t>
         </is>
       </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="500">
       <c r="A500" t="inlineStr">
@@ -6290,6 +6410,11 @@
           <t>534</t>
         </is>
       </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1B3, 2A, 2B1, 2B2, 3A, 3B1A1, 3B1A2, 3B1B, 3B2, 4</t>
+        </is>
+      </c>
     </row>
     <row r="501">
       <c r="A501" t="inlineStr">
@@ -6297,6 +6422,11 @@
           <t>535</t>
         </is>
       </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2A, 2B, 3A1, 3A2, 3B, 4, 5, 6A, 6B, 6C, 6D, 6E, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="502">
       <c r="A502" t="inlineStr">
@@ -6304,6 +6434,11 @@
           <t>536</t>
         </is>
       </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 2</t>
+        </is>
+      </c>
     </row>
     <row r="503">
       <c r="A503" t="inlineStr">
@@ -6311,6 +6446,11 @@
           <t>537</t>
         </is>
       </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="504">
       <c r="A504" t="inlineStr">
@@ -6318,6 +6458,11 @@
           <t>538</t>
         </is>
       </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>10, 1A1, 1A2, 1A3, 1A4, 1A5, 1A6, 1B, 1C, 1D, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="505">
       <c r="A505" t="inlineStr">
@@ -6325,6 +6470,11 @@
           <t>539</t>
         </is>
       </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>1TO5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="506">
       <c r="A506" t="inlineStr">
@@ -6332,6 +6482,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G1, 1G2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="507">
       <c r="A507" t="inlineStr">
@@ -6339,6 +6494,11 @@
           <t>540</t>
         </is>
       </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="508">
       <c r="A508" t="inlineStr">
@@ -6346,6 +6506,11 @@
           <t>541A</t>
         </is>
       </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="509">
       <c r="A509" t="inlineStr">
@@ -6353,6 +6518,11 @@
           <t>541B</t>
         </is>
       </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2A3, 2A4, 2A5, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="510">
       <c r="A510" t="inlineStr">
@@ -6360,6 +6530,11 @@
           <t>542A</t>
         </is>
       </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A1, 1A2, 1D, 2, 20, 21, 22, 23, 24, 25, 26, 3A1, 3A2A1, 3A2B1, 3B1A, 3B1A1, 3B1B1A2, 3B1B1B, 3B1B2, 3B2A1A, 3B2A1B, 3B2A2A, 3B2A3A1, 3B2A3B, 3B2B, 3B2C1A, 3B2C1B, 3B2C2A, 3B2C2B, 4, 5, 6A1, 6A2, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="511">
       <c r="A511" t="inlineStr">
@@ -6367,6 +6542,11 @@
           <t>542B</t>
         </is>
       </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="512">
       <c r="A512" t="inlineStr">
@@ -6374,6 +6554,11 @@
           <t>543</t>
         </is>
       </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>1, 2, 3A1A, 3A1B, 3A2, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="513">
       <c r="A513" t="inlineStr">
@@ -6381,6 +6566,11 @@
           <t>544</t>
         </is>
       </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15A1, 15A2, 15B, 16, 17, 18, 1A1, 1A2, 1B, 2A, 2B1, 2B2, 2B3, 3, 4A1A, 4A1B, 4A1C, 4A1D1, 4A1D2, 4A2, 4A3, 4B1A1A, 4B1A2, 4B1B, 4B2, 5A1A1, 5A1A1A1A1, 5A1A1A1B, 5A1A1B2, 5A1A2A, 5A1A2B, 5A1A3, 5A1B, 5A2A1, 5A2B, 5B1, 5B2, 6, 7A, 7B, 7C1, 7C2, 8A, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="514">
       <c r="A514" t="inlineStr">
@@ -6388,6 +6578,11 @@
           <t>545</t>
         </is>
       </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1A1, 2B1A2, 2B1A3, 2B1B, 2B2, 3A1A, 3A1B, 3A1C, 3A1D, 3A2, 3A3, 3A4, 3A5, 3A6, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="515">
       <c r="A515" t="inlineStr">
@@ -6395,6 +6590,11 @@
           <t>546</t>
         </is>
       </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="516">
       <c r="A516" t="inlineStr">
@@ -6402,6 +6602,11 @@
           <t>547A</t>
         </is>
       </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>1, 10, 2A, 2B, 3A, 3B, 4, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="517">
       <c r="A517" t="inlineStr">
@@ -6409,6 +6614,11 @@
           <t>547B</t>
         </is>
       </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="518">
       <c r="A518" t="inlineStr">
@@ -6416,6 +6626,11 @@
           <t>548</t>
         </is>
       </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A1, 3A2, 3B, 3C, 4, 5A1, 5A2, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="519">
       <c r="A519" t="inlineStr">
@@ -6423,6 +6638,11 @@
           <t>549</t>
         </is>
       </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>1, 2A1A1, 2A1A2, 2A1B, 2A2, 2A3, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="520">
       <c r="A520" t="inlineStr">
@@ -6430,6 +6650,11 @@
           <t>55</t>
         </is>
       </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="521">
       <c r="A521" t="inlineStr">
@@ -6437,6 +6662,11 @@
           <t>550</t>
         </is>
       </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="522">
       <c r="A522" t="inlineStr">
@@ -6444,6 +6674,11 @@
           <t>551</t>
         </is>
       </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>1, 2, 3A1A, 3A1B1, 3A1B2, 3A2A, 3A2B, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="523">
       <c r="A523" t="inlineStr">
@@ -6451,6 +6686,11 @@
           <t>552A</t>
         </is>
       </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="524">
       <c r="A524" t="inlineStr">
@@ -6458,6 +6698,11 @@
           <t>552B</t>
         </is>
       </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="525">
       <c r="A525" t="inlineStr">
@@ -6465,6 +6710,11 @@
           <t>553A</t>
         </is>
       </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="526">
       <c r="A526" t="inlineStr">
@@ -6472,6 +6722,11 @@
           <t>553B</t>
         </is>
       </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="527">
       <c r="A527" t="inlineStr">
@@ -6479,6 +6734,11 @@
           <t>554</t>
         </is>
       </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="528">
       <c r="A528" t="inlineStr">
@@ -6486,6 +6746,11 @@
           <t>555</t>
         </is>
       </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="529">
       <c r="A529" t="inlineStr">
@@ -6493,6 +6758,11 @@
           <t>556</t>
         </is>
       </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="530">
       <c r="A530" t="inlineStr">
@@ -6500,6 +6770,11 @@
           <t>557</t>
         </is>
       </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="531">
       <c r="A531" t="inlineStr">
@@ -6507,6 +6782,11 @@
           <t>558</t>
         </is>
       </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="532">
       <c r="A532" t="inlineStr">
@@ -6514,6 +6794,11 @@
           <t>559A</t>
         </is>
       </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="533">
       <c r="A533" t="inlineStr">
@@ -6521,6 +6806,11 @@
           <t>559B</t>
         </is>
       </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="534">
       <c r="A534" t="inlineStr">
@@ -6528,6 +6818,11 @@
           <t>56</t>
         </is>
       </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="535">
       <c r="A535" t="inlineStr">
@@ -6535,6 +6830,11 @@
           <t>560A</t>
         </is>
       </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="536">
       <c r="A536" t="inlineStr">
@@ -6542,6 +6842,11 @@
           <t>560B</t>
         </is>
       </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="537">
       <c r="A537" t="inlineStr">
@@ -6549,6 +6854,11 @@
           <t>561</t>
         </is>
       </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="538">
       <c r="A538" t="inlineStr">
@@ -6556,6 +6866,11 @@
           <t>562</t>
         </is>
       </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12A1A, 12A1B, 12A2, 12B, 13, 14, 15A, 15B, 15C, 15D, 16, 17A, 17B, 18, 19, 2, 20, 21A, 21B, 21C, 21D, 21E, 21F, 21G, 22, 23, 24A, 24B, 25A, 25B, 26A1, 26A2, 26B1, 26B2, 27A1A1, 27A1A2, 27A2, 27B1A, 27B1A2, 27B1A3, 27B1B, 27B1C, 27B2, 28, 29, 3, 30A1, 30A2, 30A3, 30A4, 30A5, 31, 32, 33, 34A1, 34A2, 34B, 34C, 35A, 35B, 36, 37, 38, 39, 42A, 42B, 43A, 43B1, 43B2, 44, 45, 46, 47, 48, 49, 4A, 4B, 4C, 4D, 4E, 4F, 4G, 5A, 5B, 5C, 5D, 5E, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="539">
       <c r="A539" t="inlineStr">
@@ -6563,6 +6878,11 @@
           <t>563</t>
         </is>
       </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2A1A1, 2A1A2, 2A1B, 2A1C1A1, 2A1C2, 2A1C3A, 2A1C3B, 2A1C3C, 2A1C3D, 2A2A, 2A2B, 2B, 2C1, 2C2, 2C3, 2D1A1, 2D1A2, 2D1B1A, 2D1B1B, 2D1B2A, 2D2, 2E1, 2E2A1, 2E2A2, 2E2B, 3A1A1A, 3A1B, 3A1C, 3A1D, 3A1E, 3A1F, 3A2, 3A3A1, 3A3A2, 3A3A3, 3A3A4, 3A3B, 3A3C, 3B, 3C1A, 3C1A2, 3C1B, 3C1C, 3C1D, 3C2, 4, 40, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="540">
       <c r="A540" t="inlineStr">
@@ -6570,6 +6890,11 @@
           <t>564</t>
         </is>
       </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="541">
       <c r="A541" t="inlineStr">
@@ -6577,6 +6902,11 @@
           <t>565</t>
         </is>
       </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1A, 2A1B, 2A1C, 2A2, 2B1A1A1, 2B1A1B, 2B1A2, 2B1A3, 2B1B, 2B2, 2B3A1, 2B3A2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="542">
       <c r="A542" t="inlineStr">
@@ -6584,6 +6914,11 @@
           <t>566</t>
         </is>
       </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="543">
       <c r="A543" t="inlineStr">
@@ -6591,6 +6926,11 @@
           <t>567</t>
         </is>
       </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>1, 2A1A, 2A1B, 2A2, 2A3, 2B1A, 2B1B, 2B2, 2C1, 2C2, 2C3</t>
+        </is>
+      </c>
     </row>
     <row r="544">
       <c r="A544" t="inlineStr">
@@ -6598,6 +6938,11 @@
           <t>568</t>
         </is>
       </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="545">
       <c r="A545" t="inlineStr">
@@ -6605,6 +6950,11 @@
           <t>569</t>
         </is>
       </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="546">
       <c r="A546" t="inlineStr">
@@ -6612,6 +6962,11 @@
           <t>57</t>
         </is>
       </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B, 1C, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="547">
       <c r="A547" t="inlineStr">
@@ -6619,6 +6974,11 @@
           <t>570</t>
         </is>
       </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="548">
       <c r="A548" t="inlineStr">
@@ -6626,6 +6986,11 @@
           <t>571</t>
         </is>
       </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="549">
       <c r="A549" t="inlineStr">
@@ -6633,6 +6998,11 @@
           <t>572</t>
         </is>
       </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 2D</t>
+        </is>
+      </c>
     </row>
     <row r="550">
       <c r="A550" t="inlineStr">
@@ -6640,6 +7010,11 @@
           <t>573</t>
         </is>
       </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1A1A, 2A1A2, 2A1B, 2A2, 2B1, 2B2, 2C, 3A, 3B1, 3B2, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="551">
       <c r="A551" t="inlineStr">
@@ -6647,6 +7022,11 @@
           <t>574</t>
         </is>
       </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1B, 2A, 2B, 3A1A1, 3A1A2A, 3A1A2B, 3A1A3A, 3A1A3B, 3A1B, 3A2, 3B, 4A1A1, 4A1A2, 4A1B1A, 4A1B1B, 4A1B2, 4A2, 4B1A1, 4B1A2, 4B1B, 4B1C, 4B2A1, 4B2A2, 4B2B, 4C1, 4C2A, 4C2B, 4C3</t>
+        </is>
+      </c>
     </row>
     <row r="552">
       <c r="A552" t="inlineStr">
@@ -6654,6 +7034,11 @@
           <t>575</t>
         </is>
       </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="553">
       <c r="A553" t="inlineStr">
@@ -6661,6 +7046,11 @@
           <t>576</t>
         </is>
       </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="554">
       <c r="A554" t="inlineStr">
@@ -6668,6 +7058,11 @@
           <t>577</t>
         </is>
       </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 1A1A, 1A2A, 1A2B, 1B, 2A, 2B1A, 2B1A2, 2B1B, 2B2A, 2B2B, 2B2C, 2B2D1, 2B2D2, 2B2D3, 2B2D4, 3, 4A, 4B1, 4B2, 5A1, 5A2, 5B1A, 5B1B, 5B1C, 5B2A, 5B2B, 5B3A1, 5B3A2, 5B3B1, 5B3B2, 6A1A, 6A1B1, 6A1B2, 6A1B3, 6A2A, 6A2B, 6A2C1, 6A2C2, 6A2C3, 6A2D, 6A2E1, 6A2E2, 6A2E3, 6A2E4, 6A2E5, 6A2E6, 6A2E7, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="555">
       <c r="A555" t="inlineStr">
@@ -6675,6 +7070,11 @@
           <t>578</t>
         </is>
       </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="556">
       <c r="A556" t="inlineStr">
@@ -6682,6 +7082,11 @@
           <t>579</t>
         </is>
       </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>10, 12, 1A1A1A, 1A1A1A1A, 1A2, 2A2, 2B1A1, 2B1B, 2B2, 2C1A, 2C1B, 2C2, 2C3A, 2C3B1, 2C3B2, 3, 4, 5A, 5B, 5C, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="557">
       <c r="A557" t="inlineStr">
@@ -6689,6 +7094,11 @@
           <t>58</t>
         </is>
       </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1A, 2A1B, 2A1C, 2A2, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="558">
       <c r="A558" t="inlineStr">
@@ -6696,6 +7106,11 @@
           <t>580</t>
         </is>
       </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2A, 1A2B, 1A2C, 1B, 2A1A, 2A1B, 2A2A, 2A2B, 2B1, 2B2, 2B3, 2C1, 2C2A, 2C2B1, 2C2B2</t>
+        </is>
+      </c>
     </row>
     <row r="559">
       <c r="A559" t="inlineStr">
@@ -6703,6 +7118,11 @@
           <t>581</t>
         </is>
       </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>12, 13, 17, 18A, 18B, 18C, 19, 1A1, 1A2, 1A3, 1B1A1, 1B1B, 1B1C1, 1B1C2, 1B2, 1B3, 1B4, 1C1A1, 1C1B, 1C2A, 1C2B, 1C3, 1D1A, 1D1B, 1D2, 20, 21, 23, 27, 28, 29, 2A1A1, 2A1A1A1A1B, 2A1A1A2, 2A1A1B1, 2A1A1C, 2A1A1D, 2A1A2A, 2A1A2B, 2A1A3, 2A1B, 2A1C, 2A1D, 2A1E, 30, 31, 32A1, 32B, 33, 34, 35A, 35B, 36, 37, 38, 39, 3A1A1, 3A1A1A1B, 3A1A1A2, 3A1A1B, 3A1B, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 4A, 4B, 50, 51, 52, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="560">
       <c r="A560" t="inlineStr">
@@ -6710,6 +7130,11 @@
           <t>582</t>
         </is>
       </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="561">
       <c r="A561" t="inlineStr">
@@ -6717,6 +7142,11 @@
           <t>583</t>
         </is>
       </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2A, 1A2B, 1A3, 1A4, 1A5, 1A6, 1C1, 1C2A1A1, 1C2A1B, 1C2A2, 1C2B, 1C2C, 1C2D1B, 1C2D2A1, 1C2E, 2A1, 2A2, 2B1A, 2B1B, 2B2, 2C, 2D1, 2D2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="562">
       <c r="A562" t="inlineStr">
@@ -6724,6 +7154,11 @@
           <t>584</t>
         </is>
       </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="563">
       <c r="A563" t="inlineStr">
@@ -6731,6 +7166,11 @@
           <t>585A</t>
         </is>
       </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="564">
       <c r="A564" t="inlineStr">
@@ -6738,6 +7178,11 @@
           <t>585B</t>
         </is>
       </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24A, 24B, 25, 26, 27, 28, 29, 2A, 2B, 2C, 2C1A1A, 2C1A1A2, 2C1A1B1, 2C1A2, 2C1B1, 2C1B2, 2C2, 2C3, 2C4, 2C5, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 3A10, 3A1A1, 3A1A1A1B, 3A1A1A2, 3A1A1A3, 3A1A1B, 3A1A2, 3A1B1, 3A1B2, 3A2, 3A3, 3A4, 3A5, 3A6, 3B1, 3B2, 40, 41, 42, 43, 44, 45, 46, 4A, 4B, 5, 6, 6A, 6B, 6C, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="565">
       <c r="A565" t="inlineStr">
@@ -6745,6 +7190,11 @@
           <t>586</t>
         </is>
       </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>11, 12, 13, 14, 15, 16, 17, 18, 19, 1A1A, 1A1B, 1A2, 1B, 1B2A, 1B2B1, 1B2B1A1, 1B2B2, 1B2C, 1C1, 1C1A, 1C2, 1C2A1, 1C2A1B, 1C2A2, 1C2B, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A1A, 2A1B, 2A2, 2A3, 2B, 30, 31, 3A1A1, 3A1B, 3A2, 3B, 4A1A, 4A1B, 5, 6, 7A, 7B1, 7B2, 7B3, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="566">
       <c r="A566" t="inlineStr">
@@ -6752,6 +7202,11 @@
           <t>587A</t>
         </is>
       </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="567">
       <c r="A567" t="inlineStr">
@@ -6759,6 +7214,11 @@
           <t>587B</t>
         </is>
       </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A, 1B, 20, 21, 22, 23, 24, 25, 26, 27A, 27B, 27C, 28A, 28B, 28C, 29, 2A1A, 2A1B, 2A2, 2B, 30, 31, 32, 33, 34, 35, 36, 37, 38A1, 38A2, 38B, 39, 3A, 3A1A, 3A2, 3B, 40, 41, 42, 43, 4A1A, 4A2, 4A31, 4B1A1A1, 4B1A2, 4B1B1, 4B1B2, 4B2, 4B3, 4C1A1, 4C1B1, 4C1B2, 4C2, 4C3, 5, 6A1, 6A2, 6A3, 6A4, 6B1A, 6B1B, 6B2, 6C1, 6C2, 6C3, 6C4, 6D, 7A1A1A, 7A2, 7A3, 7A4, 7B1A, 7B1B, 7B1C, 7B1C2, 7B2, 8, 9A1, 9A2, 9B1A, 9B1B, 9B2A, 9B2B, 9B2C, 9B2D</t>
+        </is>
+      </c>
     </row>
     <row r="568">
       <c r="A568" t="inlineStr">
@@ -6766,6 +7226,11 @@
           <t>588</t>
         </is>
       </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1C, 1A2, 1C1A, 1C1B, 1C2, 2, 3A1A, 3A1B, 3A2A, 3A2B, 3A3, 3B1A, 3B1B, 3B2, 3C, 3D, 3E1, 3E2, 4A, 4B, 4C1A1, 4C1A2, 4C1B, 4C2, 5A1A, 5A1B1A1, 5A1B1A2, 5A1B2, 5A2, 5A3A, 5A3B, 5B, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="569">
       <c r="A569" t="inlineStr">
@@ -6773,6 +7238,11 @@
           <t>589</t>
         </is>
       </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="570">
       <c r="A570" t="inlineStr">
@@ -6780,6 +7250,11 @@
           <t>59</t>
         </is>
       </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="571">
       <c r="A571" t="inlineStr">
@@ -6787,6 +7262,11 @@
           <t>590</t>
         </is>
       </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B1, 10B2, 10B3A1A, 11, 12, 13A1, 13A2, 13B, 13C1, 13C2, 14A1A, 14A1B, 14A2, 15, 16, 17, 18A, 18B, 19A, 19B, 2, 20A, 20A1B, 20B, 21, 22A, 22B, 23A, 23B, 24, 25A, 25B, 25C, 25D1, 25D2, 25E1, 25E2, 26, 27A1, 27A2A, 27A2B, 27B, 28, 29, 3, 30, 31, 35, 36, 37, 38, 39, 4, 40, 5, 6, 7A1A, 7A1B1, 7A1B3, 7A1B4, 7A2, 7B, 8A, 8B1, 8B2, 8C, 8D, 9</t>
+        </is>
+      </c>
     </row>
     <row r="572">
       <c r="A572" t="inlineStr">
@@ -6794,6 +7274,11 @@
           <t>591</t>
         </is>
       </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A1A, 2A1B, 2A2, 2A3, 2B, 3A1A1, 3A1A2, 3A1B, 3A2, 3A3A, 3A3B, 3A3C, 3A4, 3A5A, 3A5B, 3A5C, 3A5D, 3A5E, 3A5F, 3A5G, 3A6, 3A7, 3B1, 3B2, 3B3, 3B4, 3B5, 3B6, 3B7, 4A1A, 4A1B, 4A2, 4B1, 4B2, 4C1A, 4C1B, 4C1C, 4C1D, 4C2, 5A1, 5A2, 5B, 6A, 6B, 6C, 6D, 6E, 7A1, 7A2, 7A3, 7B, 7C, 7D, 7E, 8</t>
+        </is>
+      </c>
     </row>
     <row r="573">
       <c r="A573" t="inlineStr">
@@ -6801,6 +7286,11 @@
           <t>592A</t>
         </is>
       </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>1, 2A1A, 2A1B, 2A1C, 2A1D, 2A1E1, 2A1E2, 2A1F1, 2A1F2, 2A1G1, 2A1G2, 2A1H, 2A1J, 2A1K, 2A1LA, 2A1LB, 2A2A1A, 2A2A1B1, 2A2A1B2, 2A2A1C, 2A2A2, 2A2A3, 2A2A4, 2A2A5, 2A2B, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="574">
       <c r="A574" t="inlineStr">
@@ -6808,6 +7298,11 @@
           <t>592B</t>
         </is>
       </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B1, 1B2, 1C1, 1C2A, 1C2B, 1C3A1, 1C3A2, 1C3A3, 1C3A4, 1C3A5, 1C3A6, 1C3A7, 1C3B, 1C4A, 1C4B1, 1C4B2, 1C4C, 1C5, 1C6A1, 1C6B, 1C7, 2, 3, 4, 5, 6A</t>
+        </is>
+      </c>
     </row>
     <row r="575">
       <c r="A575" t="inlineStr">
@@ -6815,6 +7310,11 @@
           <t>592C</t>
         </is>
       </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="576">
       <c r="A576" t="inlineStr">
@@ -6822,6 +7322,11 @@
           <t>593</t>
         </is>
       </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>1A1A1, 1A1A2, 1A1B, 1A2A, 1A2B, 1A2C1A, 1A2C1C, 1A2C2, 1A2D, 1B1, 1B2, 1C1, 1C2A, 1C2B, 2A, 2B1, 2B2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="577">
       <c r="A577" t="inlineStr">
@@ -6829,6 +7334,11 @@
           <t>594</t>
         </is>
       </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1A, 2A1B, 2A1C, 2A2, 2B1, 2B2, 2B3, 3A1A1A, 3A1B, 3A2, 3B, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="578">
       <c r="A578" t="inlineStr">
@@ -6836,11 +7346,21 @@
           <t>595</t>
         </is>
       </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 1A1A, 1A1B, 1A1C, 1A2, 1A3, 1A4, 1A5, 1B, 2A1, 2A2, 2B, 2C1A1A, 2C1A1B, 2C1B, 2C1C, 2C2, 3B1A1A, 5A1, 5A2A1, 5A2B, 5A2C, 5B1, 5B2, 6A1A1, 6A1A2B, 6A1A3, 6A1A4, 6A1B, 6A2A, 6A3, 6A4, 6A5, 6A6, 6B, 6C1A1, 6C1B1, 6C1B2, 6C1B3, 6C2, 6C3A, 6C3B, 6C4, 6C5, 6C6, 6C7, 7A1, 7A2, 7B1, 7B2, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="579">
       <c r="A579" t="inlineStr">
         <is>
           <t>596</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B1, 1A1B2, 1A1C, 1A1D, 1A1E, 1A1F, 1A1G, 1A1H, 1A1I1, 1A1I2, 1A1J, 1A1K, 1A1L, 1A1M, 1A2A, 1A2B, 1A3A, 1A3B, 1B, 1B1A, 1B1B1A, 1B1B1B, 1B1B2, 1B1C1, 1B1C2A1A, 1B1C2A1A2, 1B1C2A1B, 1B1C2A1C, 1B1C2A2, 1B1C2B, 1B1C2C, 1B2, 1B3, 1B4, 2A1A, 2A1B, 2A2, 2B, 3A1A, 3A1B, 3A2, 3B1A1, 3B1A2, 3B1B1, 3B1B2, 3B2, 3C1A1A, 3C1A1B1A, 3C1A2, 3C1B, 3C1C1, 3C1C2A, 3C1C2B, 3C2, 4, 5, 6, 7, 8</t>
         </is>
       </c>
     </row>

</xml_diff>